<commit_message>
xlsx: Add formatted sheet for quali schedule
</commit_message>
<xml_diff>
--- a/bracket.xlsx
+++ b/bracket.xlsx
@@ -5,15 +5,16 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="attendance" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="quali_schedule" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="quali_score" sheetId="3" state="visible" r:id="rId4"/>
-    <sheet name="quali_results" sheetId="4" state="visible" r:id="rId5"/>
-    <sheet name="knockout_score" sheetId="5" state="visible" r:id="rId6"/>
-    <sheet name="score_slip" sheetId="6" state="visible" r:id="rId7"/>
+    <sheet name="quali_schedule_format" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="quali_score" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="quali_results" sheetId="5" state="visible" r:id="rId6"/>
+    <sheet name="knockout_score" sheetId="6" state="visible" r:id="rId7"/>
+    <sheet name="score_slip" sheetId="7" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -416,20 +417,47 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEEEEE"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
@@ -454,24 +482,10 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right style="thin"/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top/>
-      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
@@ -521,7 +535,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -570,55 +584,63 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -626,63 +648,55 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -690,7 +704,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -703,6 +721,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFEEEEEE"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -712,7 +790,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G1000"/>
-  <sheetFormatPr defaultColWidth="13.171875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.75"/>
@@ -4556,13 +4634,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:O1000"/>
-  <sheetFormatPr defaultColWidth="13.171875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="3" style="1" width="10.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="9.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="16" style="1" width="12.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="12.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="999" style="1" width="11.52"/>
   </cols>
   <sheetData>
     <row r="1" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4590,8 +4669,8 @@
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="17" s="12" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" s="10" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" s="4" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -4619,7 +4698,7 @@
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="45" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -5598,8 +5677,1580 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="13.171875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AMJ1000"/>
+  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="3" style="1" width="10.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="9.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="12.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="999" style="1" width="11.52"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="ALK1" s="1"/>
+      <c r="ALL1" s="1"/>
+      <c r="ALM1" s="1"/>
+      <c r="ALN1" s="1"/>
+      <c r="ALO1" s="1"/>
+      <c r="ALP1" s="1"/>
+      <c r="ALQ1" s="1"/>
+      <c r="ALR1" s="1"/>
+      <c r="ALS1" s="1"/>
+      <c r="ALT1" s="1"/>
+      <c r="ALU1" s="1"/>
+      <c r="ALV1" s="1"/>
+      <c r="ALW1" s="1"/>
+      <c r="ALX1" s="1"/>
+      <c r="ALY1" s="1"/>
+      <c r="ALZ1" s="1"/>
+      <c r="AMA1" s="1"/>
+      <c r="AMB1" s="1"/>
+      <c r="AMC1" s="1"/>
+      <c r="AMD1" s="1"/>
+      <c r="AME1" s="1"/>
+      <c r="AMF1" s="1"/>
+      <c r="AMG1" s="1"/>
+      <c r="AMH1" s="1"/>
+      <c r="AMI1" s="1"/>
+      <c r="AMJ1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" s="10" customFormat="true" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="12"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="12"/>
+      <c r="L16" s="12"/>
+      <c r="M16" s="12"/>
+      <c r="N16" s="12"/>
+      <c r="ALK16" s="1"/>
+      <c r="ALL16" s="1"/>
+      <c r="ALM16" s="1"/>
+      <c r="ALN16" s="1"/>
+      <c r="ALO16" s="1"/>
+      <c r="ALP16" s="1"/>
+      <c r="ALQ16" s="1"/>
+      <c r="ALR16" s="1"/>
+      <c r="ALS16" s="1"/>
+      <c r="ALT16" s="1"/>
+      <c r="ALU16" s="1"/>
+      <c r="ALV16" s="1"/>
+      <c r="ALW16" s="1"/>
+      <c r="ALX16" s="1"/>
+      <c r="ALY16" s="1"/>
+      <c r="ALZ16" s="1"/>
+      <c r="AMA16" s="1"/>
+      <c r="AMB16" s="1"/>
+      <c r="AMC16" s="1"/>
+      <c r="AMD16" s="1"/>
+      <c r="AME16" s="1"/>
+      <c r="AMF16" s="1"/>
+      <c r="AMG16" s="1"/>
+      <c r="AMH16" s="1"/>
+      <c r="AMI16" s="1"/>
+      <c r="AMJ16" s="1"/>
+    </row>
+    <row r="17" s="14" customFormat="true" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="13"/>
+      <c r="J17" s="13"/>
+      <c r="K17" s="13"/>
+      <c r="L17" s="13"/>
+      <c r="M17" s="13"/>
+      <c r="N17" s="13"/>
+      <c r="ALK17" s="1"/>
+      <c r="ALL17" s="1"/>
+      <c r="ALM17" s="1"/>
+      <c r="ALN17" s="1"/>
+      <c r="ALO17" s="1"/>
+      <c r="ALP17" s="1"/>
+      <c r="ALQ17" s="1"/>
+      <c r="ALR17" s="1"/>
+      <c r="ALS17" s="1"/>
+      <c r="ALT17" s="1"/>
+      <c r="ALU17" s="1"/>
+      <c r="ALV17" s="1"/>
+      <c r="ALW17" s="1"/>
+      <c r="ALX17" s="1"/>
+      <c r="ALY17" s="1"/>
+      <c r="ALZ17" s="1"/>
+      <c r="AMA17" s="1"/>
+      <c r="AMB17" s="1"/>
+      <c r="AMC17" s="1"/>
+      <c r="AMD17" s="1"/>
+      <c r="AME17" s="1"/>
+      <c r="AMF17" s="1"/>
+      <c r="AMG17" s="1"/>
+      <c r="AMH17" s="1"/>
+      <c r="AMI17" s="1"/>
+      <c r="AMJ17" s="1"/>
+    </row>
+    <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="15"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
+      <c r="I18" s="15"/>
+      <c r="J18" s="15"/>
+      <c r="K18" s="15"/>
+      <c r="L18" s="15"/>
+      <c r="M18" s="15"/>
+      <c r="N18" s="15"/>
+    </row>
+    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13"/>
+      <c r="L19" s="13"/>
+      <c r="M19" s="13"/>
+      <c r="N19" s="13"/>
+    </row>
+    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="15"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+      <c r="L20" s="15"/>
+      <c r="M20" s="15"/>
+      <c r="N20" s="15"/>
+    </row>
+    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="13"/>
+      <c r="J21" s="13"/>
+      <c r="K21" s="13"/>
+      <c r="L21" s="13"/>
+      <c r="M21" s="13"/>
+      <c r="N21" s="13"/>
+    </row>
+    <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="15"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="15"/>
+      <c r="I22" s="15"/>
+      <c r="J22" s="15"/>
+      <c r="K22" s="15"/>
+      <c r="L22" s="15"/>
+      <c r="M22" s="15"/>
+      <c r="N22" s="15"/>
+    </row>
+    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="13"/>
+      <c r="J23" s="13"/>
+      <c r="K23" s="13"/>
+      <c r="L23" s="13"/>
+      <c r="M23" s="13"/>
+      <c r="N23" s="13"/>
+    </row>
+    <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="15"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
+      <c r="I24" s="15"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="15"/>
+      <c r="L24" s="15"/>
+      <c r="M24" s="15"/>
+      <c r="N24" s="15"/>
+    </row>
+    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="13"/>
+      <c r="H25" s="13"/>
+      <c r="I25" s="13"/>
+      <c r="J25" s="13"/>
+      <c r="K25" s="13"/>
+      <c r="L25" s="13"/>
+      <c r="M25" s="13"/>
+      <c r="N25" s="13"/>
+    </row>
+    <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="15"/>
+      <c r="B26" s="15"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="15"/>
+      <c r="I26" s="15"/>
+      <c r="J26" s="15"/>
+      <c r="K26" s="15"/>
+      <c r="L26" s="15"/>
+      <c r="M26" s="15"/>
+      <c r="N26" s="15"/>
+    </row>
+    <row r="27" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="13"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
+      <c r="H27" s="13"/>
+      <c r="I27" s="13"/>
+      <c r="J27" s="13"/>
+      <c r="K27" s="13"/>
+      <c r="L27" s="13"/>
+      <c r="M27" s="13"/>
+      <c r="N27" s="13"/>
+    </row>
+    <row r="28" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="15"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
+      <c r="I28" s="15"/>
+      <c r="J28" s="15"/>
+      <c r="K28" s="15"/>
+      <c r="L28" s="15"/>
+      <c r="M28" s="15"/>
+      <c r="N28" s="15"/>
+    </row>
+    <row r="29" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="13"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="13"/>
+      <c r="H29" s="13"/>
+      <c r="I29" s="13"/>
+      <c r="J29" s="13"/>
+      <c r="K29" s="13"/>
+      <c r="L29" s="13"/>
+      <c r="M29" s="13"/>
+      <c r="N29" s="13"/>
+    </row>
+    <row r="30" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="15"/>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="H30" s="15"/>
+      <c r="I30" s="15"/>
+      <c r="J30" s="15"/>
+      <c r="K30" s="15"/>
+      <c r="L30" s="15"/>
+      <c r="M30" s="15"/>
+      <c r="N30" s="15"/>
+    </row>
+    <row r="31" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
+      <c r="G31" s="13"/>
+      <c r="H31" s="13"/>
+      <c r="I31" s="13"/>
+      <c r="J31" s="13"/>
+      <c r="K31" s="13"/>
+      <c r="L31" s="13"/>
+      <c r="M31" s="13"/>
+      <c r="N31" s="13"/>
+    </row>
+    <row r="32" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="15"/>
+      <c r="B32" s="15"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15"/>
+      <c r="H32" s="15"/>
+      <c r="I32" s="15"/>
+      <c r="J32" s="15"/>
+      <c r="K32" s="15"/>
+      <c r="L32" s="15"/>
+      <c r="M32" s="15"/>
+      <c r="N32" s="15"/>
+    </row>
+    <row r="33" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="13"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
+      <c r="F33" s="13"/>
+      <c r="G33" s="13"/>
+      <c r="H33" s="13"/>
+      <c r="I33" s="13"/>
+      <c r="J33" s="13"/>
+      <c r="K33" s="13"/>
+      <c r="L33" s="13"/>
+      <c r="M33" s="13"/>
+      <c r="N33" s="13"/>
+    </row>
+    <row r="34" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="15"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="15"/>
+      <c r="I34" s="15"/>
+      <c r="J34" s="15"/>
+      <c r="K34" s="15"/>
+      <c r="L34" s="15"/>
+      <c r="M34" s="15"/>
+      <c r="N34" s="15"/>
+    </row>
+    <row r="35" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="13"/>
+      <c r="B35" s="13"/>
+      <c r="C35" s="13"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="13"/>
+      <c r="F35" s="13"/>
+      <c r="G35" s="13"/>
+      <c r="H35" s="13"/>
+      <c r="I35" s="13"/>
+      <c r="J35" s="13"/>
+      <c r="K35" s="13"/>
+      <c r="L35" s="13"/>
+      <c r="M35" s="13"/>
+      <c r="N35" s="13"/>
+    </row>
+    <row r="36" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="15"/>
+      <c r="B36" s="15"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="15"/>
+      <c r="I36" s="15"/>
+      <c r="J36" s="15"/>
+      <c r="K36" s="15"/>
+      <c r="L36" s="15"/>
+      <c r="M36" s="15"/>
+      <c r="N36" s="15"/>
+    </row>
+    <row r="37" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="13"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="13"/>
+      <c r="F37" s="13"/>
+      <c r="G37" s="13"/>
+      <c r="H37" s="13"/>
+      <c r="I37" s="13"/>
+      <c r="J37" s="13"/>
+      <c r="K37" s="13"/>
+      <c r="L37" s="13"/>
+      <c r="M37" s="13"/>
+      <c r="N37" s="13"/>
+    </row>
+    <row r="38" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="15"/>
+      <c r="B38" s="15"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="15"/>
+      <c r="F38" s="15"/>
+      <c r="G38" s="15"/>
+      <c r="H38" s="15"/>
+      <c r="I38" s="15"/>
+      <c r="J38" s="15"/>
+      <c r="K38" s="15"/>
+      <c r="L38" s="15"/>
+      <c r="M38" s="15"/>
+      <c r="N38" s="15"/>
+    </row>
+    <row r="39" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="13"/>
+      <c r="B39" s="13"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="13"/>
+      <c r="F39" s="13"/>
+      <c r="G39" s="13"/>
+      <c r="H39" s="13"/>
+      <c r="I39" s="13"/>
+      <c r="J39" s="13"/>
+      <c r="K39" s="13"/>
+      <c r="L39" s="13"/>
+      <c r="M39" s="13"/>
+      <c r="N39" s="13"/>
+    </row>
+    <row r="40" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="15"/>
+      <c r="B40" s="15"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="15"/>
+      <c r="G40" s="15"/>
+      <c r="H40" s="15"/>
+      <c r="I40" s="15"/>
+      <c r="J40" s="15"/>
+      <c r="K40" s="15"/>
+      <c r="L40" s="15"/>
+      <c r="M40" s="15"/>
+      <c r="N40" s="15"/>
+    </row>
+    <row r="41" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="13"/>
+      <c r="B41" s="13"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="13"/>
+      <c r="F41" s="13"/>
+      <c r="G41" s="13"/>
+      <c r="H41" s="13"/>
+      <c r="I41" s="13"/>
+      <c r="J41" s="13"/>
+      <c r="K41" s="13"/>
+      <c r="L41" s="13"/>
+      <c r="M41" s="13"/>
+      <c r="N41" s="13"/>
+    </row>
+    <row r="42" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="15"/>
+      <c r="B42" s="15"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="15"/>
+      <c r="F42" s="15"/>
+      <c r="G42" s="15"/>
+      <c r="H42" s="15"/>
+      <c r="I42" s="15"/>
+      <c r="J42" s="15"/>
+      <c r="K42" s="15"/>
+      <c r="L42" s="15"/>
+      <c r="M42" s="15"/>
+      <c r="N42" s="15"/>
+    </row>
+    <row r="43" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="13"/>
+      <c r="B43" s="13"/>
+      <c r="C43" s="13"/>
+      <c r="D43" s="13"/>
+      <c r="E43" s="13"/>
+      <c r="F43" s="13"/>
+      <c r="G43" s="13"/>
+      <c r="H43" s="13"/>
+      <c r="I43" s="13"/>
+      <c r="J43" s="13"/>
+      <c r="K43" s="13"/>
+      <c r="L43" s="13"/>
+      <c r="M43" s="13"/>
+      <c r="N43" s="13"/>
+    </row>
+    <row r="44" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="15"/>
+      <c r="B44" s="15"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="15"/>
+      <c r="G44" s="15"/>
+      <c r="H44" s="15"/>
+      <c r="I44" s="15"/>
+      <c r="J44" s="15"/>
+      <c r="K44" s="15"/>
+      <c r="L44" s="15"/>
+      <c r="M44" s="15"/>
+      <c r="N44" s="15"/>
+    </row>
+    <row r="45" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="16"/>
+      <c r="B45" s="16"/>
+      <c r="C45" s="16"/>
+      <c r="D45" s="16"/>
+      <c r="E45" s="16"/>
+      <c r="F45" s="16"/>
+      <c r="G45" s="16"/>
+      <c r="H45" s="16"/>
+      <c r="I45" s="16"/>
+      <c r="J45" s="16"/>
+      <c r="K45" s="16"/>
+      <c r="L45" s="16"/>
+      <c r="M45" s="16"/>
+      <c r="N45" s="16"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="81" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="92" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="93" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="94" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="95" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="96" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="97" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="98" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="99" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="100" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="101" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="102" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="103" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="104" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="105" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="106" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="107" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="108" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="109" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="110" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="111" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="112" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="113" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="114" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="115" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="116" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="117" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="118" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="119" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="120" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="121" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="122" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="123" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="124" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="125" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="126" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="127" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="128" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="129" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="130" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="131" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="132" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="133" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="134" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="135" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="136" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="137" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="138" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="139" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="140" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="141" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="142" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="143" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="144" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="145" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="146" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="147" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="148" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="149" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="150" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="151" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="152" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="153" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="154" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="155" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="156" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="157" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="158" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="159" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="160" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="161" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="162" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="163" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="164" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="165" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="166" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="167" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="168" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="169" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="170" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="171" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="172" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="173" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="174" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="175" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="176" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="177" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="178" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="179" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="180" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="181" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="182" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="183" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="184" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="185" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="186" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="187" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="188" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="189" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="190" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="191" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="192" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="193" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="194" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="195" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="196" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="197" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="198" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="199" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="200" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="201" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="202" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="203" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="204" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="205" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="206" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="207" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="208" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="209" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="210" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="211" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="212" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="213" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="214" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="215" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="216" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="217" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="218" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="219" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="220" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="221" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="222" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="223" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="224" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="225" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="226" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="227" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="228" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="229" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="230" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="231" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="232" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="233" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="234" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="235" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="236" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="237" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="238" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="239" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="240" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="241" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="242" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="243" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="244" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="245" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="246" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="247" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="248" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="249" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="250" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="251" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="252" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="253" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="254" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="255" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="256" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="257" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="258" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="259" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="260" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="261" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="262" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="263" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="264" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="265" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="266" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="267" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="268" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="269" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="270" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="271" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="272" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="273" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="274" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="275" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="276" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="277" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="278" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="279" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="280" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="281" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="282" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="283" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="284" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="285" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="286" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="287" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="288" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="289" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="290" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="291" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="292" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="293" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="294" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="295" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="296" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="297" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="298" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="299" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="300" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="301" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="302" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="303" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="304" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="305" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="306" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="307" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="308" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="309" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="310" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="311" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="312" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="313" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="314" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="315" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="316" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="317" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="318" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="319" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="320" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="321" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="322" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="323" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="324" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="325" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="326" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="327" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="328" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="329" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="330" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="331" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="332" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="333" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="334" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="335" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="336" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="337" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="338" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="339" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="340" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="341" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="342" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="343" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="344" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="345" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="346" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="347" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="348" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="349" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="350" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="351" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="352" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="353" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="354" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="355" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="356" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="357" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="358" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="359" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="360" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="361" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="362" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="363" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="364" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="365" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="366" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="367" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="368" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="369" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="370" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="371" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="372" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="373" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="374" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="375" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="376" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="377" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="378" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="379" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="380" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="381" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="382" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="383" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="384" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="385" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="386" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="387" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="388" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="389" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="390" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="391" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="392" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="393" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="394" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="395" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="396" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="397" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="398" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="399" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="400" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="401" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="402" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="403" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="404" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="405" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="406" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="407" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="408" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="409" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="410" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="411" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="412" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="413" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="414" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="415" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="416" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="417" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="418" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="419" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="420" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="421" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="422" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="423" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="424" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="425" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="426" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="427" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="428" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="429" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="430" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="431" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="432" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="433" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="434" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="435" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="436" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="437" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="438" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="439" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="440" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="441" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="442" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="443" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="444" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="445" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="446" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="447" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="448" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="449" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="450" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="451" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="452" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="453" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="454" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="455" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="456" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="457" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="458" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="459" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="460" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="461" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="462" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="463" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="464" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="465" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="466" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="467" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="468" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="469" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="470" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="471" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="472" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="473" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="474" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="475" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="476" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="477" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="478" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="479" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="480" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="481" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="482" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="483" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="484" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="485" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="486" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="487" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="488" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="489" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="490" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="491" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="492" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="493" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="494" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="495" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="496" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="497" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="498" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="499" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="500" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="501" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="502" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="503" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="504" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="505" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="506" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="507" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="508" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="509" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="510" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="511" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="512" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="513" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="514" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="515" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="516" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="517" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="518" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="519" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="520" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="521" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="522" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="523" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="524" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="525" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="526" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="527" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="528" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="529" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="530" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="531" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="532" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="533" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="534" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="535" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="536" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="537" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="538" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="539" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="540" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="541" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="542" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="543" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="544" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="545" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="546" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="547" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="548" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="549" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="550" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="551" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="552" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="553" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="554" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="555" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="556" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="557" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="558" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="559" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="560" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="561" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="562" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="563" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="564" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="565" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="566" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="567" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="568" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="569" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="570" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="571" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="572" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="573" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="574" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="575" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="576" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="577" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="578" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="579" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="580" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="581" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="582" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="583" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="584" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="585" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="586" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="587" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="588" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="589" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="590" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="591" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="592" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="593" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="594" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="595" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="596" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="597" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="598" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="599" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="600" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="601" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="602" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="603" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="604" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="605" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="606" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="607" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="608" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="609" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="610" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="611" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="612" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="613" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="614" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="615" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="616" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="617" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="618" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="619" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="620" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="621" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="622" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="623" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="624" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="625" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="626" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="627" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="628" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="629" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="630" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="631" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="632" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="633" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="634" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="635" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="636" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="637" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="638" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="639" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="640" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="641" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="642" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="643" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="644" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="645" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="646" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="647" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="648" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="649" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="650" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="651" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="652" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="653" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="654" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="655" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="656" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="657" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="658" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="659" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="660" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="661" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="662" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="663" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="664" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="665" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="666" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="667" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="668" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="669" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="670" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="671" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="672" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="673" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="674" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="675" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="676" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="677" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="678" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="679" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="680" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="681" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="682" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="683" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="684" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="685" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="686" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="687" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="688" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="689" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="690" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="691" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="692" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="693" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="694" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="695" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="696" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="697" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="698" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="699" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="700" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="701" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="702" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="703" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="704" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="705" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="706" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="707" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="708" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="709" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="710" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="711" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="712" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="713" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="714" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="715" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="716" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="717" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="718" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="719" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="720" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="721" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="722" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="723" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="724" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="725" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="726" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="727" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="728" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="729" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="730" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="731" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="732" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="733" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="734" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="735" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="736" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="737" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="738" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="739" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="740" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="741" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="742" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="743" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="744" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="745" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="746" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="747" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="748" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="749" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="750" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="751" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="752" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="753" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="754" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="755" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="756" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="757" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="758" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="759" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="760" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="761" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="762" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="763" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="764" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="765" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="766" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="767" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="768" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="769" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="770" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="771" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="772" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="773" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="774" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="775" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="776" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="777" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="778" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="779" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="780" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="781" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="782" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="783" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="784" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="785" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="786" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="787" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="788" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="789" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="790" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="791" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="792" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="793" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="794" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="795" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="796" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="797" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="798" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="799" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="800" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="801" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="802" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="803" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="804" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="805" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="806" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="807" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="808" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="809" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="810" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="811" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="812" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="813" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="814" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="815" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="816" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="817" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="818" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="819" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="820" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="821" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="822" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="823" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="824" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="825" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="826" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="827" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="828" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="829" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="830" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="831" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="832" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="833" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="834" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="835" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="836" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="837" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="838" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="839" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="840" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="841" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="842" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="843" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="844" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="845" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="846" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="847" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="848" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="849" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="850" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="851" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="852" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="853" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="854" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="855" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="856" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="857" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="858" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="859" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="860" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="861" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="862" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="863" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="864" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="865" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="866" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="867" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="868" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="869" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="870" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="871" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="872" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="873" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="874" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="875" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="876" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="877" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="878" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="879" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="880" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="881" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="882" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="883" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="884" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="885" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="886" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="887" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="888" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="889" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="890" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="891" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="892" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="893" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="894" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="895" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="896" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="897" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="898" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="899" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="900" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="901" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="902" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="903" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="904" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="905" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="906" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="907" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="908" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="909" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="910" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="911" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="912" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="913" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="914" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="915" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="916" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="917" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="918" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="919" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="920" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="921" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="922" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="923" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="924" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="925" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="926" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="927" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="928" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="929" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="930" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="931" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="932" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="933" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="934" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="935" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="936" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="937" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="938" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="939" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="940" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="941" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="942" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="943" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="944" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="945" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="946" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="947" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="948" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="949" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="950" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="951" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="952" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="953" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="954" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="955" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="956" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="957" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="958" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="959" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="960" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="961" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="962" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="963" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="964" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="965" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="966" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="967" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="968" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="969" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="970" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="971" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="972" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="973" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="974" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="975" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="976" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="977" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="978" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="979" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="980" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="981" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="982" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="983" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="984" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="985" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="986" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="987" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="988" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="989" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="990" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="991" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="992" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="993" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="994" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="995" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="996" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="997" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="998" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="999" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1000" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="N1:O1"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.5"/>
@@ -5613,34 +7264,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="10" style="1" width="11.5"/>
   </cols>
   <sheetData>
-    <row r="1" s="13" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3"/>
-      <c r="B1" s="3"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="3"/>
-      <c r="R1" s="3"/>
-      <c r="S1" s="3"/>
-      <c r="T1" s="3"/>
-      <c r="U1" s="3"/>
-      <c r="V1" s="3"/>
-      <c r="W1" s="3"/>
-      <c r="X1" s="3"/>
-      <c r="Y1" s="3"/>
-      <c r="Z1" s="3"/>
-    </row>
+    <row r="1" s="3" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -6651,19 +8275,19 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C39"/>
-  <sheetFormatPr defaultColWidth="11.83984375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.94140625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="9" width="11.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="9" width="11.52"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="11" min="5" style="9" width="11.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1022" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="5" style="9" width="11.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1022" style="1" width="11.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -6857,13 +8481,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:T86"/>
-  <sheetFormatPr defaultColWidth="11.83984375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.94140625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="11.69"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25.52"/>
@@ -6878,42 +8502,42 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="16"/>
-      <c r="N1" s="15"/>
-      <c r="O1" s="15"/>
-      <c r="P1" s="15"/>
-      <c r="Q1" s="15"/>
-      <c r="R1" s="16"/>
-      <c r="S1" s="16"/>
-      <c r="T1" s="17"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="18"/>
+      <c r="O1" s="18"/>
+      <c r="P1" s="18"/>
+      <c r="Q1" s="18"/>
+      <c r="R1" s="19"/>
+      <c r="S1" s="19"/>
+      <c r="T1" s="20"/>
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14"/>
-      <c r="B2" s="18" t="n">
+      <c r="A2" s="17"/>
+      <c r="B2" s="21" t="n">
         <f aca="false">VLOOKUP("a1", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C2" s="18" t="n">
+      <c r="C2" s="21" t="n">
         <f aca="false">VLOOKUP("a1", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
@@ -6921,104 +8545,104 @@
       <c r="K2" s="6"/>
       <c r="L2" s="6"/>
       <c r="M2" s="6"/>
-      <c r="T2" s="20"/>
+      <c r="T2" s="23"/>
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14"/>
-      <c r="B3" s="21" t="n">
+      <c r="A3" s="17"/>
+      <c r="B3" s="24" t="n">
         <f aca="false">VLOOKUP("c2", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C3" s="21" t="n">
+      <c r="C3" s="24" t="n">
         <f aca="false">VLOOKUP("c2", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="23"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="26"/>
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
       <c r="K3" s="6"/>
       <c r="L3" s="6"/>
       <c r="M3" s="6"/>
-      <c r="T3" s="20"/>
+      <c r="T3" s="23"/>
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14"/>
+      <c r="A4" s="17"/>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
-      <c r="G4" s="24"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="26"/>
-      <c r="J4" s="26"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="25"/>
-      <c r="T4" s="20"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="28"/>
+      <c r="T4" s="23"/>
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14"/>
+      <c r="A5" s="17"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
-      <c r="G5" s="24"/>
+      <c r="G5" s="27"/>
       <c r="H5" s="5"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="24"/>
-      <c r="T5" s="20"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
+      <c r="K5" s="25"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="25"/>
+      <c r="N5" s="27"/>
+      <c r="T5" s="23"/>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14"/>
-      <c r="B6" s="18" t="n">
+      <c r="A6" s="17"/>
+      <c r="B6" s="21" t="n">
         <f aca="false">VLOOKUP("a2", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C6" s="18" t="n">
+      <c r="C6" s="21" t="n">
         <f aca="false">VLOOKUP("a2", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="28"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="29"/>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="6"/>
       <c r="L6" s="6"/>
       <c r="M6" s="6"/>
-      <c r="N6" s="24"/>
+      <c r="N6" s="27"/>
       <c r="P6" s="5"/>
       <c r="Q6" s="5"/>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
-      <c r="T6" s="29"/>
+      <c r="T6" s="30"/>
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14"/>
-      <c r="B7" s="21" t="n">
+      <c r="A7" s="17"/>
+      <c r="B7" s="24" t="n">
         <f aca="false">VLOOKUP("c1", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="24" t="n">
         <f aca="false">VLOOKUP("c1", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
@@ -7026,45 +8650,45 @@
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
       <c r="M7" s="6"/>
-      <c r="N7" s="24"/>
-      <c r="O7" s="25"/>
-      <c r="P7" s="26"/>
-      <c r="Q7" s="26"/>
-      <c r="R7" s="19"/>
-      <c r="S7" s="19"/>
-      <c r="T7" s="19"/>
+      <c r="N7" s="27"/>
+      <c r="O7" s="28"/>
+      <c r="P7" s="21"/>
+      <c r="Q7" s="21"/>
+      <c r="R7" s="22"/>
+      <c r="S7" s="22"/>
+      <c r="T7" s="22"/>
     </row>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14"/>
-      <c r="N8" s="24"/>
-      <c r="P8" s="27"/>
-      <c r="Q8" s="27"/>
-      <c r="R8" s="22"/>
-      <c r="S8" s="22"/>
-      <c r="T8" s="22"/>
+      <c r="A8" s="17"/>
+      <c r="N8" s="27"/>
+      <c r="P8" s="24"/>
+      <c r="Q8" s="24"/>
+      <c r="R8" s="25"/>
+      <c r="S8" s="25"/>
+      <c r="T8" s="25"/>
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14"/>
-      <c r="N9" s="24"/>
+      <c r="A9" s="17"/>
+      <c r="N9" s="27"/>
       <c r="P9" s="5"/>
       <c r="Q9" s="5"/>
       <c r="R9" s="6"/>
       <c r="S9" s="6"/>
-      <c r="T9" s="29"/>
+      <c r="T9" s="30"/>
     </row>
     <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14"/>
-      <c r="B10" s="18" t="n">
+      <c r="A10" s="17"/>
+      <c r="B10" s="21" t="n">
         <f aca="false">VLOOKUP("b1", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C10" s="18" t="n">
+      <c r="C10" s="21" t="n">
         <f aca="false">VLOOKUP("b1", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
@@ -7072,113 +8696,113 @@
       <c r="K10" s="6"/>
       <c r="L10" s="6"/>
       <c r="M10" s="6"/>
-      <c r="N10" s="24"/>
-      <c r="O10" s="25"/>
-      <c r="P10" s="26"/>
-      <c r="Q10" s="26"/>
-      <c r="R10" s="19"/>
-      <c r="S10" s="19"/>
-      <c r="T10" s="19"/>
+      <c r="N10" s="27"/>
+      <c r="O10" s="28"/>
+      <c r="P10" s="21"/>
+      <c r="Q10" s="21"/>
+      <c r="R10" s="22"/>
+      <c r="S10" s="22"/>
+      <c r="T10" s="22"/>
     </row>
     <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14"/>
-      <c r="B11" s="18" t="n">
+      <c r="A11" s="17"/>
+      <c r="B11" s="21" t="n">
         <f aca="false">VLOOKUP("d2", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C11" s="18" t="n">
+      <c r="C11" s="21" t="n">
         <f aca="false">VLOOKUP("d2", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="23"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="26"/>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
       <c r="K11" s="6"/>
       <c r="L11" s="6"/>
       <c r="M11" s="6"/>
-      <c r="N11" s="24"/>
-      <c r="P11" s="27"/>
-      <c r="Q11" s="27"/>
-      <c r="R11" s="22"/>
-      <c r="S11" s="22"/>
-      <c r="T11" s="22"/>
+      <c r="N11" s="27"/>
+      <c r="P11" s="24"/>
+      <c r="Q11" s="24"/>
+      <c r="R11" s="25"/>
+      <c r="S11" s="25"/>
+      <c r="T11" s="25"/>
     </row>
     <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14"/>
+      <c r="A12" s="17"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
       <c r="F12" s="6"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="25"/>
-      <c r="I12" s="26"/>
-      <c r="J12" s="26"/>
-      <c r="K12" s="19"/>
-      <c r="L12" s="19"/>
-      <c r="M12" s="19"/>
-      <c r="N12" s="28"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="21"/>
+      <c r="J12" s="21"/>
+      <c r="K12" s="22"/>
+      <c r="L12" s="22"/>
+      <c r="M12" s="22"/>
+      <c r="N12" s="29"/>
       <c r="P12" s="5"/>
       <c r="Q12" s="5"/>
       <c r="R12" s="6"/>
       <c r="S12" s="6"/>
-      <c r="T12" s="29"/>
+      <c r="T12" s="30"/>
     </row>
     <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14"/>
+      <c r="A13" s="17"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
-      <c r="G13" s="24"/>
+      <c r="G13" s="27"/>
       <c r="H13" s="5"/>
-      <c r="I13" s="27"/>
-      <c r="J13" s="27"/>
-      <c r="K13" s="22"/>
-      <c r="L13" s="22"/>
-      <c r="M13" s="22"/>
-      <c r="T13" s="20"/>
+      <c r="I13" s="24"/>
+      <c r="J13" s="24"/>
+      <c r="K13" s="25"/>
+      <c r="L13" s="25"/>
+      <c r="M13" s="25"/>
+      <c r="T13" s="23"/>
     </row>
     <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14"/>
-      <c r="B14" s="18" t="n">
+      <c r="A14" s="17"/>
+      <c r="B14" s="21" t="n">
         <f aca="false">VLOOKUP("b2", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C14" s="18" t="n">
+      <c r="C14" s="21" t="n">
         <f aca="false">VLOOKUP("b2", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="28"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="29"/>
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
       <c r="K14" s="6"/>
       <c r="L14" s="6"/>
       <c r="M14" s="6"/>
-      <c r="T14" s="20"/>
+      <c r="T14" s="23"/>
     </row>
     <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="14"/>
-      <c r="B15" s="21" t="n">
+      <c r="A15" s="17"/>
+      <c r="B15" s="24" t="n">
         <f aca="false">VLOOKUP("d1", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C15" s="21" t="n">
+      <c r="C15" s="24" t="n">
         <f aca="false">VLOOKUP("d1", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
@@ -7186,75 +8810,75 @@
       <c r="K15" s="6"/>
       <c r="L15" s="6"/>
       <c r="M15" s="6"/>
-      <c r="T15" s="20"/>
+      <c r="T15" s="23"/>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14"/>
-      <c r="T16" s="20"/>
+      <c r="A16" s="17"/>
+      <c r="T16" s="23"/>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14"/>
-      <c r="B17" s="30"/>
-      <c r="C17" s="30"/>
-      <c r="D17" s="31"/>
-      <c r="E17" s="31"/>
-      <c r="F17" s="31"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="30"/>
-      <c r="I17" s="30"/>
-      <c r="J17" s="30"/>
-      <c r="K17" s="31"/>
-      <c r="L17" s="31"/>
-      <c r="M17" s="31"/>
-      <c r="N17" s="30"/>
-      <c r="O17" s="30"/>
-      <c r="P17" s="30"/>
-      <c r="Q17" s="30"/>
-      <c r="R17" s="31"/>
-      <c r="S17" s="31"/>
-      <c r="T17" s="32"/>
+      <c r="A17" s="17"/>
+      <c r="B17" s="31"/>
+      <c r="C17" s="31"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="32"/>
+      <c r="G17" s="31"/>
+      <c r="H17" s="31"/>
+      <c r="I17" s="31"/>
+      <c r="J17" s="31"/>
+      <c r="K17" s="32"/>
+      <c r="L17" s="32"/>
+      <c r="M17" s="32"/>
+      <c r="N17" s="31"/>
+      <c r="O17" s="31"/>
+      <c r="P17" s="31"/>
+      <c r="Q17" s="31"/>
+      <c r="R17" s="32"/>
+      <c r="S17" s="32"/>
+      <c r="T17" s="33"/>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="15"/>
-      <c r="O18" s="15"/>
-      <c r="P18" s="15"/>
-      <c r="Q18" s="15"/>
-      <c r="R18" s="16"/>
-      <c r="S18" s="16"/>
-      <c r="T18" s="17"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="19"/>
+      <c r="L18" s="19"/>
+      <c r="M18" s="19"/>
+      <c r="N18" s="18"/>
+      <c r="O18" s="18"/>
+      <c r="P18" s="18"/>
+      <c r="Q18" s="18"/>
+      <c r="R18" s="19"/>
+      <c r="S18" s="19"/>
+      <c r="T18" s="20"/>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14"/>
-      <c r="T19" s="20"/>
+      <c r="A19" s="17"/>
+      <c r="T19" s="23"/>
     </row>
     <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="14"/>
-      <c r="B20" s="18" t="n">
+      <c r="A20" s="17"/>
+      <c r="B20" s="21" t="n">
         <f aca="false">VLOOKUP("a3", quali_results!$A$1:$C40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C20" s="18" t="n">
+      <c r="C20" s="21" t="n">
         <f aca="false">VLOOKUP("a3", quali_results!$A$1:$C40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
       <c r="G20" s="5"/>
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
@@ -7262,104 +8886,104 @@
       <c r="K20" s="6"/>
       <c r="L20" s="6"/>
       <c r="M20" s="6"/>
-      <c r="T20" s="20"/>
+      <c r="T20" s="23"/>
     </row>
     <row r="21" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14"/>
-      <c r="B21" s="21" t="n">
+      <c r="A21" s="17"/>
+      <c r="B21" s="24" t="n">
         <f aca="false">VLOOKUP("c4", quali_results!$A$1:$C40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C21" s="21" t="n">
+      <c r="C21" s="24" t="n">
         <f aca="false">VLOOKUP("c4", quali_results!$A$1:$C40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="23"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="26"/>
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
       <c r="J21" s="5"/>
       <c r="K21" s="6"/>
       <c r="L21" s="6"/>
       <c r="M21" s="6"/>
-      <c r="T21" s="20"/>
+      <c r="T21" s="23"/>
     </row>
     <row r="22" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14"/>
+      <c r="A22" s="17"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="26"/>
-      <c r="J22" s="26"/>
-      <c r="K22" s="19"/>
-      <c r="L22" s="19"/>
-      <c r="M22" s="19"/>
-      <c r="N22" s="25"/>
-      <c r="T22" s="20"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="28"/>
+      <c r="I22" s="21"/>
+      <c r="J22" s="21"/>
+      <c r="K22" s="22"/>
+      <c r="L22" s="22"/>
+      <c r="M22" s="22"/>
+      <c r="N22" s="28"/>
+      <c r="T22" s="23"/>
     </row>
     <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14"/>
+      <c r="A23" s="17"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
       <c r="F23" s="6"/>
-      <c r="G23" s="24"/>
+      <c r="G23" s="27"/>
       <c r="H23" s="5"/>
-      <c r="I23" s="27"/>
-      <c r="J23" s="27"/>
-      <c r="K23" s="22"/>
-      <c r="L23" s="22"/>
-      <c r="M23" s="22"/>
-      <c r="N23" s="24"/>
-      <c r="T23" s="20"/>
+      <c r="I23" s="24"/>
+      <c r="J23" s="24"/>
+      <c r="K23" s="25"/>
+      <c r="L23" s="25"/>
+      <c r="M23" s="25"/>
+      <c r="N23" s="27"/>
+      <c r="T23" s="23"/>
     </row>
     <row r="24" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14"/>
-      <c r="B24" s="18" t="n">
+      <c r="A24" s="17"/>
+      <c r="B24" s="21" t="n">
         <f aca="false">VLOOKUP("a4", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C24" s="18" t="n">
+      <c r="C24" s="21" t="n">
         <f aca="false">VLOOKUP("a4", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="28"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="22"/>
+      <c r="G24" s="29"/>
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
       <c r="J24" s="5"/>
       <c r="K24" s="6"/>
       <c r="L24" s="6"/>
       <c r="M24" s="6"/>
-      <c r="N24" s="24"/>
+      <c r="N24" s="27"/>
       <c r="P24" s="5"/>
       <c r="Q24" s="5"/>
       <c r="R24" s="6"/>
       <c r="S24" s="6"/>
-      <c r="T24" s="29"/>
+      <c r="T24" s="30"/>
     </row>
     <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14"/>
-      <c r="B25" s="21" t="n">
+      <c r="A25" s="17"/>
+      <c r="B25" s="24" t="n">
         <f aca="false">VLOOKUP("c3", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C25" s="21" t="n">
+      <c r="C25" s="24" t="n">
         <f aca="false">VLOOKUP("c3", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="25"/>
       <c r="G25" s="5"/>
       <c r="H25" s="5"/>
       <c r="I25" s="5"/>
@@ -7367,45 +8991,45 @@
       <c r="K25" s="6"/>
       <c r="L25" s="6"/>
       <c r="M25" s="6"/>
-      <c r="N25" s="24"/>
-      <c r="O25" s="25"/>
-      <c r="P25" s="26"/>
-      <c r="Q25" s="26"/>
-      <c r="R25" s="19"/>
-      <c r="S25" s="19"/>
-      <c r="T25" s="19"/>
+      <c r="N25" s="27"/>
+      <c r="O25" s="28"/>
+      <c r="P25" s="21"/>
+      <c r="Q25" s="21"/>
+      <c r="R25" s="22"/>
+      <c r="S25" s="22"/>
+      <c r="T25" s="22"/>
     </row>
     <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="14"/>
-      <c r="N26" s="24"/>
-      <c r="P26" s="27"/>
-      <c r="Q26" s="27"/>
-      <c r="R26" s="22"/>
-      <c r="S26" s="22"/>
-      <c r="T26" s="22"/>
+      <c r="A26" s="17"/>
+      <c r="N26" s="27"/>
+      <c r="P26" s="24"/>
+      <c r="Q26" s="24"/>
+      <c r="R26" s="25"/>
+      <c r="S26" s="25"/>
+      <c r="T26" s="25"/>
     </row>
     <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="14"/>
-      <c r="N27" s="24"/>
+      <c r="A27" s="17"/>
+      <c r="N27" s="27"/>
       <c r="P27" s="5"/>
       <c r="Q27" s="5"/>
       <c r="R27" s="6"/>
       <c r="S27" s="6"/>
-      <c r="T27" s="29"/>
+      <c r="T27" s="30"/>
     </row>
     <row r="28" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="14"/>
-      <c r="B28" s="18" t="n">
+      <c r="A28" s="17"/>
+      <c r="B28" s="21" t="n">
         <f aca="false">VLOOKUP("b3", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C28" s="18" t="n">
+      <c r="C28" s="21" t="n">
         <f aca="false">VLOOKUP("b3", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="22"/>
       <c r="G28" s="5"/>
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
@@ -7413,113 +9037,113 @@
       <c r="K28" s="6"/>
       <c r="L28" s="6"/>
       <c r="M28" s="6"/>
-      <c r="N28" s="24"/>
-      <c r="O28" s="25"/>
-      <c r="P28" s="26"/>
-      <c r="Q28" s="26"/>
-      <c r="R28" s="19"/>
-      <c r="S28" s="19"/>
-      <c r="T28" s="19"/>
+      <c r="N28" s="27"/>
+      <c r="O28" s="28"/>
+      <c r="P28" s="21"/>
+      <c r="Q28" s="21"/>
+      <c r="R28" s="22"/>
+      <c r="S28" s="22"/>
+      <c r="T28" s="22"/>
     </row>
     <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14"/>
-      <c r="B29" s="21" t="n">
+      <c r="A29" s="17"/>
+      <c r="B29" s="24" t="n">
         <f aca="false">VLOOKUP("d4", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C29" s="21" t="n">
+      <c r="C29" s="24" t="n">
         <f aca="false">VLOOKUP("d4", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D29" s="22"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="22"/>
-      <c r="G29" s="23"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="26"/>
       <c r="H29" s="5"/>
       <c r="I29" s="5"/>
       <c r="J29" s="5"/>
       <c r="K29" s="6"/>
       <c r="L29" s="6"/>
       <c r="M29" s="6"/>
-      <c r="N29" s="24"/>
-      <c r="P29" s="27"/>
-      <c r="Q29" s="27"/>
-      <c r="R29" s="22"/>
-      <c r="S29" s="22"/>
-      <c r="T29" s="22"/>
+      <c r="N29" s="27"/>
+      <c r="P29" s="24"/>
+      <c r="Q29" s="24"/>
+      <c r="R29" s="25"/>
+      <c r="S29" s="25"/>
+      <c r="T29" s="25"/>
     </row>
     <row r="30" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="14"/>
+      <c r="A30" s="17"/>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
       <c r="D30" s="6"/>
       <c r="E30" s="6"/>
       <c r="F30" s="6"/>
-      <c r="G30" s="24"/>
-      <c r="H30" s="25"/>
-      <c r="I30" s="26"/>
-      <c r="J30" s="26"/>
-      <c r="K30" s="19"/>
-      <c r="L30" s="19"/>
-      <c r="M30" s="19"/>
-      <c r="N30" s="28"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="28"/>
+      <c r="I30" s="21"/>
+      <c r="J30" s="21"/>
+      <c r="K30" s="22"/>
+      <c r="L30" s="22"/>
+      <c r="M30" s="22"/>
+      <c r="N30" s="29"/>
       <c r="P30" s="5"/>
       <c r="Q30" s="5"/>
       <c r="R30" s="6"/>
       <c r="S30" s="6"/>
-      <c r="T30" s="29"/>
+      <c r="T30" s="30"/>
     </row>
     <row r="31" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="14"/>
+      <c r="A31" s="17"/>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
       <c r="D31" s="6"/>
       <c r="E31" s="6"/>
       <c r="F31" s="6"/>
-      <c r="G31" s="24"/>
+      <c r="G31" s="27"/>
       <c r="H31" s="5"/>
-      <c r="I31" s="27"/>
-      <c r="J31" s="27"/>
-      <c r="K31" s="22"/>
-      <c r="L31" s="22"/>
-      <c r="M31" s="22"/>
-      <c r="T31" s="20"/>
+      <c r="I31" s="24"/>
+      <c r="J31" s="24"/>
+      <c r="K31" s="25"/>
+      <c r="L31" s="25"/>
+      <c r="M31" s="25"/>
+      <c r="T31" s="23"/>
     </row>
     <row r="32" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="14"/>
-      <c r="B32" s="18" t="n">
+      <c r="A32" s="17"/>
+      <c r="B32" s="21" t="n">
         <f aca="false">VLOOKUP("b4", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C32" s="18" t="n">
+      <c r="C32" s="21" t="n">
         <f aca="false">VLOOKUP("b4", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="28"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="29"/>
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
       <c r="J32" s="5"/>
       <c r="K32" s="6"/>
       <c r="L32" s="6"/>
       <c r="M32" s="6"/>
-      <c r="T32" s="20"/>
+      <c r="T32" s="23"/>
     </row>
     <row r="33" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="14"/>
-      <c r="B33" s="21" t="n">
+      <c r="A33" s="17"/>
+      <c r="B33" s="24" t="n">
         <f aca="false">VLOOKUP("d3", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C33" s="21" t="n">
+      <c r="C33" s="24" t="n">
         <f aca="false">VLOOKUP("d3", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D33" s="22"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="22"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="25"/>
       <c r="G33" s="5"/>
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
@@ -7527,570 +9151,570 @@
       <c r="K33" s="6"/>
       <c r="L33" s="6"/>
       <c r="M33" s="6"/>
-      <c r="T33" s="20"/>
+      <c r="T33" s="23"/>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="14"/>
-      <c r="T34" s="20"/>
+      <c r="A34" s="17"/>
+      <c r="T34" s="23"/>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="14"/>
-      <c r="B35" s="30"/>
-      <c r="C35" s="30"/>
-      <c r="D35" s="31"/>
-      <c r="E35" s="31"/>
-      <c r="F35" s="31"/>
-      <c r="G35" s="30"/>
-      <c r="H35" s="30"/>
-      <c r="I35" s="30"/>
-      <c r="J35" s="30"/>
-      <c r="K35" s="31"/>
-      <c r="L35" s="31"/>
-      <c r="M35" s="31"/>
-      <c r="N35" s="30"/>
-      <c r="O35" s="30"/>
-      <c r="P35" s="30"/>
-      <c r="Q35" s="30"/>
-      <c r="R35" s="31"/>
-      <c r="S35" s="31"/>
-      <c r="T35" s="32"/>
+      <c r="A35" s="17"/>
+      <c r="B35" s="31"/>
+      <c r="C35" s="31"/>
+      <c r="D35" s="32"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="32"/>
+      <c r="G35" s="31"/>
+      <c r="H35" s="31"/>
+      <c r="I35" s="31"/>
+      <c r="J35" s="31"/>
+      <c r="K35" s="32"/>
+      <c r="L35" s="32"/>
+      <c r="M35" s="32"/>
+      <c r="N35" s="31"/>
+      <c r="O35" s="31"/>
+      <c r="P35" s="31"/>
+      <c r="Q35" s="31"/>
+      <c r="R35" s="32"/>
+      <c r="S35" s="32"/>
+      <c r="T35" s="33"/>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="14" t="s">
+      <c r="A36" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="I36" s="15"/>
-      <c r="J36" s="15"/>
-      <c r="K36" s="16"/>
-      <c r="L36" s="16"/>
-      <c r="M36" s="16"/>
-      <c r="N36" s="15"/>
-      <c r="O36" s="15"/>
-      <c r="P36" s="15"/>
-      <c r="Q36" s="15"/>
-      <c r="R36" s="16"/>
-      <c r="S36" s="16"/>
-      <c r="T36" s="17"/>
+      <c r="I36" s="18"/>
+      <c r="J36" s="18"/>
+      <c r="K36" s="19"/>
+      <c r="L36" s="19"/>
+      <c r="M36" s="19"/>
+      <c r="N36" s="18"/>
+      <c r="O36" s="18"/>
+      <c r="P36" s="18"/>
+      <c r="Q36" s="18"/>
+      <c r="R36" s="19"/>
+      <c r="S36" s="19"/>
+      <c r="T36" s="20"/>
     </row>
     <row r="37" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="14"/>
+      <c r="A37" s="17"/>
       <c r="I37" s="5"/>
       <c r="J37" s="5"/>
       <c r="K37" s="6"/>
       <c r="L37" s="6"/>
       <c r="M37" s="6"/>
-      <c r="T37" s="20"/>
+      <c r="T37" s="23"/>
     </row>
     <row r="38" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="14"/>
+      <c r="A38" s="17"/>
       <c r="I38" s="5"/>
       <c r="J38" s="5"/>
       <c r="K38" s="6"/>
       <c r="L38" s="6"/>
       <c r="M38" s="6"/>
-      <c r="T38" s="20"/>
+      <c r="T38" s="23"/>
     </row>
     <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="14"/>
-      <c r="I39" s="18" t="n">
+      <c r="A39" s="17"/>
+      <c r="I39" s="21" t="n">
         <f aca="false">VLOOKUP("a5", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="J39" s="18" t="n">
+      <c r="J39" s="21" t="n">
         <f aca="false">VLOOKUP("a5", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="K39" s="19"/>
-      <c r="L39" s="19"/>
-      <c r="M39" s="19"/>
-      <c r="N39" s="25"/>
-      <c r="T39" s="20"/>
+      <c r="K39" s="22"/>
+      <c r="L39" s="22"/>
+      <c r="M39" s="22"/>
+      <c r="N39" s="28"/>
+      <c r="T39" s="23"/>
     </row>
     <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="14"/>
-      <c r="I40" s="21" t="n">
+      <c r="A40" s="17"/>
+      <c r="I40" s="24" t="n">
         <f aca="false">VLOOKUP("c5", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="J40" s="21" t="n">
+      <c r="J40" s="24" t="n">
         <f aca="false">VLOOKUP("c5", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="K40" s="22"/>
-      <c r="L40" s="22"/>
-      <c r="M40" s="22"/>
-      <c r="N40" s="24"/>
-      <c r="T40" s="20"/>
+      <c r="K40" s="25"/>
+      <c r="L40" s="25"/>
+      <c r="M40" s="25"/>
+      <c r="N40" s="27"/>
+      <c r="T40" s="23"/>
     </row>
     <row r="41" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="14"/>
+      <c r="A41" s="17"/>
       <c r="I41" s="5"/>
       <c r="J41" s="5"/>
       <c r="K41" s="6"/>
       <c r="L41" s="6"/>
       <c r="M41" s="6"/>
-      <c r="N41" s="24"/>
+      <c r="N41" s="27"/>
       <c r="P41" s="5"/>
       <c r="Q41" s="5"/>
       <c r="R41" s="6"/>
       <c r="S41" s="6"/>
-      <c r="T41" s="29"/>
+      <c r="T41" s="30"/>
     </row>
     <row r="42" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="14"/>
+      <c r="A42" s="17"/>
       <c r="I42" s="5"/>
       <c r="J42" s="5"/>
       <c r="K42" s="6"/>
       <c r="L42" s="6"/>
       <c r="M42" s="6"/>
-      <c r="N42" s="24"/>
-      <c r="O42" s="25"/>
-      <c r="P42" s="26"/>
-      <c r="Q42" s="26"/>
-      <c r="R42" s="19"/>
-      <c r="S42" s="19"/>
-      <c r="T42" s="19"/>
+      <c r="N42" s="27"/>
+      <c r="O42" s="28"/>
+      <c r="P42" s="21"/>
+      <c r="Q42" s="21"/>
+      <c r="R42" s="22"/>
+      <c r="S42" s="22"/>
+      <c r="T42" s="22"/>
     </row>
     <row r="43" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="14"/>
-      <c r="N43" s="24"/>
-      <c r="P43" s="27"/>
-      <c r="Q43" s="27"/>
-      <c r="R43" s="22"/>
-      <c r="S43" s="22"/>
-      <c r="T43" s="22"/>
+      <c r="A43" s="17"/>
+      <c r="N43" s="27"/>
+      <c r="P43" s="24"/>
+      <c r="Q43" s="24"/>
+      <c r="R43" s="25"/>
+      <c r="S43" s="25"/>
+      <c r="T43" s="25"/>
     </row>
     <row r="44" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="14"/>
-      <c r="N44" s="24"/>
+      <c r="A44" s="17"/>
+      <c r="N44" s="27"/>
       <c r="P44" s="5"/>
       <c r="Q44" s="5"/>
       <c r="R44" s="6"/>
       <c r="S44" s="6"/>
-      <c r="T44" s="29"/>
+      <c r="T44" s="30"/>
     </row>
     <row r="45" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="14"/>
+      <c r="A45" s="17"/>
       <c r="I45" s="5"/>
       <c r="J45" s="5"/>
       <c r="K45" s="6"/>
       <c r="L45" s="6"/>
       <c r="M45" s="6"/>
-      <c r="N45" s="24"/>
-      <c r="O45" s="25"/>
-      <c r="P45" s="26"/>
-      <c r="Q45" s="26"/>
-      <c r="R45" s="19"/>
-      <c r="S45" s="19"/>
-      <c r="T45" s="19"/>
+      <c r="N45" s="27"/>
+      <c r="O45" s="28"/>
+      <c r="P45" s="21"/>
+      <c r="Q45" s="21"/>
+      <c r="R45" s="22"/>
+      <c r="S45" s="22"/>
+      <c r="T45" s="22"/>
     </row>
     <row r="46" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="14"/>
+      <c r="A46" s="17"/>
       <c r="I46" s="5"/>
       <c r="J46" s="5"/>
       <c r="K46" s="6"/>
       <c r="L46" s="6"/>
       <c r="M46" s="6"/>
-      <c r="N46" s="24"/>
-      <c r="P46" s="27"/>
-      <c r="Q46" s="27"/>
-      <c r="R46" s="22"/>
-      <c r="S46" s="22"/>
-      <c r="T46" s="22"/>
+      <c r="N46" s="27"/>
+      <c r="P46" s="24"/>
+      <c r="Q46" s="24"/>
+      <c r="R46" s="25"/>
+      <c r="S46" s="25"/>
+      <c r="T46" s="25"/>
     </row>
     <row r="47" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="14"/>
-      <c r="I47" s="18" t="n">
+      <c r="A47" s="17"/>
+      <c r="I47" s="21" t="n">
         <f aca="false">VLOOKUP("b5", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="J47" s="18" t="n">
+      <c r="J47" s="21" t="n">
         <f aca="false">VLOOKUP("b5", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="K47" s="19"/>
-      <c r="L47" s="19"/>
-      <c r="M47" s="19"/>
-      <c r="N47" s="28"/>
+      <c r="K47" s="22"/>
+      <c r="L47" s="22"/>
+      <c r="M47" s="22"/>
+      <c r="N47" s="29"/>
       <c r="P47" s="5"/>
       <c r="Q47" s="5"/>
       <c r="R47" s="6"/>
       <c r="S47" s="6"/>
-      <c r="T47" s="29"/>
+      <c r="T47" s="30"/>
     </row>
     <row r="48" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="14"/>
-      <c r="I48" s="21" t="n">
+      <c r="A48" s="17"/>
+      <c r="I48" s="24" t="n">
         <f aca="false">VLOOKUP("d5", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="J48" s="21" t="n">
+      <c r="J48" s="24" t="n">
         <f aca="false">VLOOKUP("d5", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="K48" s="22"/>
-      <c r="L48" s="22"/>
-      <c r="M48" s="22"/>
-      <c r="T48" s="20"/>
+      <c r="K48" s="25"/>
+      <c r="L48" s="25"/>
+      <c r="M48" s="25"/>
+      <c r="T48" s="23"/>
     </row>
     <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="14"/>
+      <c r="A49" s="17"/>
       <c r="I49" s="5"/>
       <c r="J49" s="5"/>
       <c r="K49" s="6"/>
       <c r="L49" s="6"/>
       <c r="M49" s="6"/>
-      <c r="T49" s="20"/>
+      <c r="T49" s="23"/>
     </row>
     <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="14"/>
+      <c r="A50" s="17"/>
       <c r="I50" s="5"/>
       <c r="J50" s="5"/>
       <c r="K50" s="6"/>
       <c r="L50" s="6"/>
       <c r="M50" s="6"/>
-      <c r="T50" s="20"/>
+      <c r="T50" s="23"/>
     </row>
     <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="14"/>
-      <c r="T51" s="20"/>
+      <c r="A51" s="17"/>
+      <c r="T51" s="23"/>
     </row>
     <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="14"/>
-      <c r="B52" s="30"/>
-      <c r="C52" s="30"/>
-      <c r="D52" s="31"/>
-      <c r="E52" s="31"/>
-      <c r="F52" s="31"/>
-      <c r="G52" s="30"/>
-      <c r="H52" s="30"/>
-      <c r="I52" s="30"/>
-      <c r="J52" s="30"/>
-      <c r="K52" s="31"/>
-      <c r="L52" s="31"/>
-      <c r="M52" s="31"/>
-      <c r="N52" s="30"/>
-      <c r="O52" s="30"/>
-      <c r="P52" s="30"/>
-      <c r="Q52" s="30"/>
-      <c r="R52" s="31"/>
-      <c r="S52" s="31"/>
-      <c r="T52" s="32"/>
+      <c r="A52" s="17"/>
+      <c r="B52" s="31"/>
+      <c r="C52" s="31"/>
+      <c r="D52" s="32"/>
+      <c r="E52" s="32"/>
+      <c r="F52" s="32"/>
+      <c r="G52" s="31"/>
+      <c r="H52" s="31"/>
+      <c r="I52" s="31"/>
+      <c r="J52" s="31"/>
+      <c r="K52" s="32"/>
+      <c r="L52" s="32"/>
+      <c r="M52" s="32"/>
+      <c r="N52" s="31"/>
+      <c r="O52" s="31"/>
+      <c r="P52" s="31"/>
+      <c r="Q52" s="31"/>
+      <c r="R52" s="32"/>
+      <c r="S52" s="32"/>
+      <c r="T52" s="33"/>
     </row>
     <row r="53" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="33" t="s">
+      <c r="A53" s="34" t="s">
         <v>97</v>
       </c>
-      <c r="I53" s="15"/>
-      <c r="J53" s="15"/>
-      <c r="K53" s="16"/>
-      <c r="L53" s="16"/>
-      <c r="M53" s="16"/>
-      <c r="N53" s="15"/>
-      <c r="O53" s="15"/>
-      <c r="P53" s="15"/>
-      <c r="Q53" s="15"/>
-      <c r="R53" s="16"/>
-      <c r="S53" s="16"/>
-      <c r="T53" s="17"/>
+      <c r="I53" s="18"/>
+      <c r="J53" s="18"/>
+      <c r="K53" s="19"/>
+      <c r="L53" s="19"/>
+      <c r="M53" s="19"/>
+      <c r="N53" s="18"/>
+      <c r="O53" s="18"/>
+      <c r="P53" s="18"/>
+      <c r="Q53" s="18"/>
+      <c r="R53" s="19"/>
+      <c r="S53" s="19"/>
+      <c r="T53" s="20"/>
     </row>
     <row r="54" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="33"/>
+      <c r="A54" s="34"/>
       <c r="I54" s="5"/>
       <c r="J54" s="5"/>
       <c r="K54" s="6"/>
       <c r="L54" s="6"/>
       <c r="M54" s="6"/>
-      <c r="T54" s="20"/>
+      <c r="T54" s="23"/>
     </row>
     <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="33"/>
-      <c r="T55" s="20"/>
+      <c r="A55" s="34"/>
+      <c r="T55" s="23"/>
     </row>
     <row r="56" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="33"/>
-      <c r="T56" s="20"/>
+      <c r="A56" s="34"/>
+      <c r="T56" s="23"/>
     </row>
     <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="33"/>
-      <c r="T57" s="20"/>
+      <c r="A57" s="34"/>
+      <c r="T57" s="23"/>
     </row>
     <row r="58" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="33"/>
+      <c r="A58" s="34"/>
       <c r="P58" s="5"/>
       <c r="Q58" s="5"/>
       <c r="R58" s="6"/>
       <c r="S58" s="6"/>
-      <c r="T58" s="29"/>
+      <c r="T58" s="30"/>
     </row>
     <row r="59" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="33"/>
-      <c r="P59" s="18" t="n">
+      <c r="A59" s="34"/>
+      <c r="P59" s="21" t="n">
         <f aca="false">VLOOKUP("w1", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="Q59" s="18" t="n">
+      <c r="Q59" s="21" t="n">
         <f aca="false">VLOOKUP("w1", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="R59" s="19"/>
-      <c r="S59" s="19"/>
-      <c r="T59" s="19"/>
+      <c r="R59" s="22"/>
+      <c r="S59" s="22"/>
+      <c r="T59" s="22"/>
     </row>
     <row r="60" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="33"/>
-      <c r="P60" s="21" t="n">
+      <c r="A60" s="34"/>
+      <c r="P60" s="24" t="n">
         <f aca="false">VLOOKUP("w2", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="Q60" s="21" t="n">
+      <c r="Q60" s="24" t="n">
         <f aca="false">VLOOKUP("w2", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="R60" s="22"/>
-      <c r="S60" s="22"/>
-      <c r="T60" s="22"/>
+      <c r="R60" s="25"/>
+      <c r="S60" s="25"/>
+      <c r="T60" s="25"/>
     </row>
     <row r="61" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="33"/>
+      <c r="A61" s="34"/>
       <c r="P61" s="5"/>
       <c r="Q61" s="5"/>
       <c r="R61" s="6"/>
       <c r="S61" s="6"/>
-      <c r="T61" s="19"/>
+      <c r="T61" s="22"/>
     </row>
     <row r="62" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="33"/>
-      <c r="P62" s="18" t="n">
+      <c r="A62" s="34"/>
+      <c r="P62" s="21" t="n">
         <f aca="false">VLOOKUP("w3", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="Q62" s="18" t="n">
+      <c r="Q62" s="21" t="n">
         <f aca="false">VLOOKUP("w3", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="R62" s="19"/>
-      <c r="S62" s="19"/>
-      <c r="T62" s="19"/>
+      <c r="R62" s="22"/>
+      <c r="S62" s="22"/>
+      <c r="T62" s="22"/>
     </row>
     <row r="63" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="33"/>
-      <c r="P63" s="21" t="n">
+      <c r="A63" s="34"/>
+      <c r="P63" s="24" t="n">
         <f aca="false">VLOOKUP("w4", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="Q63" s="21" t="n">
+      <c r="Q63" s="24" t="n">
         <f aca="false">VLOOKUP("w4", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="R63" s="22"/>
-      <c r="S63" s="22"/>
-      <c r="T63" s="22"/>
+      <c r="R63" s="25"/>
+      <c r="S63" s="25"/>
+      <c r="T63" s="25"/>
     </row>
     <row r="64" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="33"/>
+      <c r="A64" s="34"/>
       <c r="P64" s="5"/>
       <c r="Q64" s="5"/>
       <c r="R64" s="6"/>
       <c r="S64" s="6"/>
-      <c r="T64" s="29"/>
+      <c r="T64" s="30"/>
     </row>
     <row r="65" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="33"/>
-      <c r="T65" s="20"/>
+      <c r="A65" s="34"/>
+      <c r="T65" s="23"/>
     </row>
     <row r="66" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="33"/>
-      <c r="T66" s="20"/>
+      <c r="A66" s="34"/>
+      <c r="T66" s="23"/>
     </row>
     <row r="67" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="33"/>
+      <c r="A67" s="34"/>
       <c r="I67" s="5"/>
       <c r="J67" s="5"/>
       <c r="K67" s="6"/>
       <c r="L67" s="6"/>
       <c r="M67" s="6"/>
-      <c r="T67" s="20"/>
+      <c r="T67" s="23"/>
     </row>
     <row r="68" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="33"/>
-      <c r="T68" s="20"/>
+      <c r="A68" s="34"/>
+      <c r="T68" s="23"/>
     </row>
     <row r="69" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="33"/>
-      <c r="B69" s="30"/>
-      <c r="C69" s="30"/>
-      <c r="D69" s="31"/>
-      <c r="E69" s="31"/>
-      <c r="F69" s="31"/>
-      <c r="G69" s="30"/>
-      <c r="H69" s="30"/>
-      <c r="I69" s="30"/>
-      <c r="J69" s="30"/>
-      <c r="K69" s="31"/>
-      <c r="L69" s="31"/>
-      <c r="M69" s="31"/>
-      <c r="N69" s="30"/>
-      <c r="O69" s="30"/>
-      <c r="P69" s="30"/>
-      <c r="Q69" s="30"/>
-      <c r="R69" s="31"/>
-      <c r="S69" s="31"/>
-      <c r="T69" s="32"/>
+      <c r="A69" s="34"/>
+      <c r="B69" s="31"/>
+      <c r="C69" s="31"/>
+      <c r="D69" s="32"/>
+      <c r="E69" s="32"/>
+      <c r="F69" s="32"/>
+      <c r="G69" s="31"/>
+      <c r="H69" s="31"/>
+      <c r="I69" s="31"/>
+      <c r="J69" s="31"/>
+      <c r="K69" s="32"/>
+      <c r="L69" s="32"/>
+      <c r="M69" s="32"/>
+      <c r="N69" s="31"/>
+      <c r="O69" s="31"/>
+      <c r="P69" s="31"/>
+      <c r="Q69" s="31"/>
+      <c r="R69" s="32"/>
+      <c r="S69" s="32"/>
+      <c r="T69" s="33"/>
     </row>
     <row r="70" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="14" t="s">
+      <c r="A70" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="P70" s="15"/>
-      <c r="Q70" s="15"/>
-      <c r="R70" s="16"/>
-      <c r="S70" s="16"/>
-      <c r="T70" s="17"/>
+      <c r="P70" s="18"/>
+      <c r="Q70" s="18"/>
+      <c r="R70" s="19"/>
+      <c r="S70" s="19"/>
+      <c r="T70" s="20"/>
     </row>
     <row r="71" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="14"/>
+      <c r="A71" s="17"/>
       <c r="I71" s="5"/>
       <c r="J71" s="5"/>
       <c r="K71" s="6"/>
       <c r="L71" s="6"/>
       <c r="M71" s="6"/>
-      <c r="T71" s="20"/>
+      <c r="T71" s="23"/>
     </row>
     <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="14"/>
-      <c r="T72" s="20"/>
+      <c r="A72" s="17"/>
+      <c r="T72" s="23"/>
     </row>
     <row r="73" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="14"/>
-      <c r="T73" s="20"/>
+      <c r="A73" s="17"/>
+      <c r="T73" s="23"/>
     </row>
     <row r="74" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="14"/>
-      <c r="T74" s="20"/>
+      <c r="A74" s="17"/>
+      <c r="T74" s="23"/>
     </row>
     <row r="75" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="14"/>
+      <c r="A75" s="17"/>
       <c r="P75" s="5"/>
       <c r="Q75" s="5"/>
       <c r="R75" s="6"/>
       <c r="S75" s="6"/>
-      <c r="T75" s="29"/>
+      <c r="T75" s="30"/>
     </row>
     <row r="76" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="14"/>
-      <c r="P76" s="18" t="n">
+      <c r="A76" s="17"/>
+      <c r="P76" s="21" t="n">
         <f aca="false">VLOOKUP("g1", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="Q76" s="18" t="n">
+      <c r="Q76" s="21" t="n">
         <f aca="false">VLOOKUP("g1", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="R76" s="19"/>
-      <c r="S76" s="19"/>
-      <c r="T76" s="19"/>
+      <c r="R76" s="22"/>
+      <c r="S76" s="22"/>
+      <c r="T76" s="22"/>
     </row>
     <row r="77" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="14"/>
-      <c r="P77" s="21" t="n">
+      <c r="A77" s="17"/>
+      <c r="P77" s="24" t="n">
         <f aca="false">VLOOKUP("g2", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="Q77" s="21" t="n">
+      <c r="Q77" s="24" t="n">
         <f aca="false">VLOOKUP("g2", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="R77" s="22"/>
-      <c r="S77" s="22"/>
-      <c r="T77" s="22"/>
+      <c r="R77" s="25"/>
+      <c r="S77" s="25"/>
+      <c r="T77" s="25"/>
     </row>
     <row r="78" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="14"/>
+      <c r="A78" s="17"/>
       <c r="P78" s="5"/>
       <c r="Q78" s="5"/>
       <c r="R78" s="6"/>
       <c r="S78" s="6"/>
-      <c r="T78" s="29"/>
+      <c r="T78" s="30"/>
     </row>
     <row r="79" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="14"/>
-      <c r="P79" s="18" t="n">
+      <c r="A79" s="17"/>
+      <c r="P79" s="21" t="n">
         <f aca="false">VLOOKUP("g3", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="Q79" s="18" t="n">
+      <c r="Q79" s="21" t="n">
         <f aca="false">VLOOKUP("g3", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="R79" s="19"/>
-      <c r="S79" s="19"/>
-      <c r="T79" s="19"/>
+      <c r="R79" s="22"/>
+      <c r="S79" s="22"/>
+      <c r="T79" s="22"/>
     </row>
     <row r="80" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="14"/>
-      <c r="P80" s="21" t="n">
+      <c r="A80" s="17"/>
+      <c r="P80" s="24" t="n">
         <f aca="false">VLOOKUP("g4", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="Q80" s="21" t="n">
+      <c r="Q80" s="24" t="n">
         <f aca="false">VLOOKUP("g4", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="R80" s="22"/>
-      <c r="S80" s="22"/>
-      <c r="T80" s="22"/>
+      <c r="R80" s="25"/>
+      <c r="S80" s="25"/>
+      <c r="T80" s="25"/>
     </row>
     <row r="81" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="14"/>
+      <c r="A81" s="17"/>
       <c r="P81" s="5"/>
       <c r="Q81" s="5"/>
       <c r="R81" s="6"/>
       <c r="S81" s="6"/>
-      <c r="T81" s="29"/>
+      <c r="T81" s="30"/>
     </row>
     <row r="82" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="14"/>
-      <c r="T82" s="20"/>
+      <c r="A82" s="17"/>
+      <c r="T82" s="23"/>
     </row>
     <row r="83" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A83" s="14"/>
-      <c r="T83" s="20"/>
+      <c r="A83" s="17"/>
+      <c r="T83" s="23"/>
     </row>
     <row r="84" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="14"/>
+      <c r="A84" s="17"/>
       <c r="I84" s="5"/>
       <c r="J84" s="5"/>
       <c r="K84" s="6"/>
       <c r="L84" s="6"/>
       <c r="M84" s="6"/>
-      <c r="T84" s="20"/>
+      <c r="T84" s="23"/>
     </row>
     <row r="85" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="14"/>
-      <c r="T85" s="20"/>
+      <c r="A85" s="17"/>
+      <c r="T85" s="23"/>
     </row>
     <row r="86" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="14"/>
-      <c r="B86" s="30"/>
-      <c r="C86" s="30"/>
-      <c r="D86" s="31"/>
-      <c r="E86" s="31"/>
-      <c r="F86" s="31"/>
-      <c r="G86" s="30"/>
-      <c r="H86" s="30"/>
-      <c r="I86" s="25"/>
-      <c r="J86" s="25"/>
-      <c r="K86" s="34"/>
-      <c r="L86" s="34"/>
-      <c r="M86" s="34"/>
-      <c r="N86" s="25"/>
-      <c r="O86" s="25"/>
-      <c r="P86" s="30"/>
-      <c r="Q86" s="30"/>
-      <c r="R86" s="31"/>
-      <c r="S86" s="31"/>
-      <c r="T86" s="32"/>
+      <c r="A86" s="17"/>
+      <c r="B86" s="31"/>
+      <c r="C86" s="31"/>
+      <c r="D86" s="32"/>
+      <c r="E86" s="32"/>
+      <c r="F86" s="32"/>
+      <c r="G86" s="31"/>
+      <c r="H86" s="31"/>
+      <c r="I86" s="28"/>
+      <c r="J86" s="28"/>
+      <c r="K86" s="35"/>
+      <c r="L86" s="35"/>
+      <c r="M86" s="35"/>
+      <c r="N86" s="28"/>
+      <c r="O86" s="28"/>
+      <c r="P86" s="31"/>
+      <c r="Q86" s="31"/>
+      <c r="R86" s="32"/>
+      <c r="S86" s="32"/>
+      <c r="T86" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -8110,13 +9734,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D27"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.92"/>
@@ -8126,156 +9750,156 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="35" t="s">
+      <c r="A6" s="36" t="s">
         <v>99</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="37" t="s">
         <v>100</v>
       </c>
-      <c r="C6" s="36"/>
-      <c r="D6" s="36"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="37"/>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="B7" s="37"/>
-      <c r="C7" s="37"/>
-      <c r="D7" s="37"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="38"/>
+      <c r="D7" s="38"/>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="35" t="s">
+      <c r="A8" s="36" t="s">
         <v>102</v>
       </c>
-      <c r="B8" s="37"/>
-      <c r="C8" s="37"/>
-      <c r="D8" s="37"/>
+      <c r="B8" s="38"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="38" t="s">
+      <c r="A9" s="39" t="s">
         <v>103</v>
       </c>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
+      <c r="B9" s="38"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="38"/>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="B10" s="39"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="40" t="s">
+      <c r="B10" s="40"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="41" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="11" s="9" customFormat="true" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="B11" s="39"/>
-      <c r="C11" s="39"/>
-      <c r="D11" s="14" t="s">
+      <c r="B11" s="40"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="17" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="12" s="9" customFormat="true" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="B12" s="39"/>
-      <c r="C12" s="39"/>
-      <c r="D12" s="14" t="s">
+      <c r="B12" s="40"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="17" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="13" s="9" customFormat="true" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="41" t="s">
+      <c r="A13" s="42" t="s">
         <v>108</v>
       </c>
-      <c r="B13" s="42"/>
-      <c r="C13" s="42"/>
-      <c r="D13" s="14" t="s">
+      <c r="B13" s="43"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="17" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="30"/>
-      <c r="B16" s="30"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
+      <c r="A16" s="31"/>
+      <c r="B16" s="31"/>
+      <c r="C16" s="31"/>
+      <c r="D16" s="31"/>
     </row>
     <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="35" t="s">
+      <c r="A20" s="36" t="s">
         <v>99</v>
       </c>
-      <c r="B20" s="36" t="s">
+      <c r="B20" s="37" t="s">
         <v>100</v>
       </c>
-      <c r="C20" s="36"/>
-      <c r="D20" s="36"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="37"/>
     </row>
     <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="35" t="s">
+      <c r="A21" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="B21" s="37"/>
-      <c r="C21" s="37"/>
-      <c r="D21" s="37"/>
+      <c r="B21" s="38"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="38"/>
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="35" t="s">
+      <c r="A22" s="36" t="s">
         <v>102</v>
       </c>
-      <c r="B22" s="37"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="37"/>
+      <c r="B22" s="38"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="38" t="s">
+      <c r="A23" s="39" t="s">
         <v>103</v>
       </c>
-      <c r="B23" s="37"/>
-      <c r="C23" s="37"/>
-      <c r="D23" s="37"/>
+      <c r="B23" s="38"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="B24" s="39"/>
-      <c r="C24" s="39"/>
-      <c r="D24" s="40" t="s">
+      <c r="B24" s="40"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="41" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="B25" s="39"/>
-      <c r="C25" s="39"/>
-      <c r="D25" s="14" t="s">
+      <c r="B25" s="40"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="17" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="14" t="s">
+      <c r="A26" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="B26" s="39"/>
-      <c r="C26" s="39"/>
-      <c r="D26" s="14" t="s">
+      <c r="B26" s="40"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="17" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="41" t="s">
+      <c r="A27" s="42" t="s">
         <v>108</v>
       </c>
-      <c r="B27" s="42"/>
-      <c r="C27" s="42"/>
-      <c r="D27" s="14" t="s">
+      <c r="B27" s="43"/>
+      <c r="C27" s="43"/>
+      <c r="D27" s="17" t="s">
         <v>108</v>
       </c>
     </row>

</xml_diff>

<commit_message>
xlsx: Single formatted sheet for quali schedule
</commit_message>
<xml_diff>
--- a/bracket.xlsx
+++ b/bracket.xlsx
@@ -5,16 +5,15 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="attendance" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="quali_schedule" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="quali_schedule_format" sheetId="3" state="visible" r:id="rId4"/>
-    <sheet name="quali_score" sheetId="4" state="visible" r:id="rId5"/>
-    <sheet name="quali_results" sheetId="5" state="visible" r:id="rId6"/>
-    <sheet name="knockout_score" sheetId="6" state="visible" r:id="rId7"/>
-    <sheet name="score_slip" sheetId="7" state="visible" r:id="rId8"/>
+    <sheet name="quali_score" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="quali_results" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="knockout_score" sheetId="5" state="visible" r:id="rId6"/>
+    <sheet name="score_slip" sheetId="6" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -580,10 +579,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -626,6 +621,10 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -708,7 +707,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -790,7 +789,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G1000"/>
-  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.30859375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.75"/>
@@ -4633,8 +4632,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:O1000"/>
-  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AMJ1000"/>
+  <sheetFormatPr defaultColWidth="13.30859375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.51"/>
@@ -4645,16 +4644,43 @@
   </cols>
   <sheetData>
     <row r="1" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="N1" s="11"/>
-      <c r="O1" s="11"/>
+      <c r="A1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="ALK1" s="1"/>
+      <c r="ALL1" s="1"/>
+      <c r="ALM1" s="1"/>
+      <c r="ALN1" s="1"/>
+      <c r="ALO1" s="1"/>
+      <c r="ALP1" s="1"/>
+      <c r="ALQ1" s="1"/>
+      <c r="ALR1" s="1"/>
+      <c r="ALS1" s="1"/>
+      <c r="ALT1" s="1"/>
+      <c r="ALU1" s="1"/>
+      <c r="ALV1" s="1"/>
+      <c r="ALW1" s="1"/>
+      <c r="ALX1" s="1"/>
+      <c r="ALY1" s="1"/>
+      <c r="ALZ1" s="1"/>
+      <c r="AMA1" s="1"/>
+      <c r="AMB1" s="1"/>
+      <c r="AMC1" s="1"/>
+      <c r="AMD1" s="1"/>
+      <c r="AME1" s="1"/>
+      <c r="AMF1" s="1"/>
+      <c r="AMG1" s="1"/>
+      <c r="AMH1" s="1"/>
+      <c r="AMI1" s="1"/>
+      <c r="AMJ1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -4669,36 +4695,538 @@
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="16" s="10" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="17" s="4" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="45" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" s="10" customFormat="true" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="11"/>
+      <c r="N16" s="11"/>
+      <c r="ALK16" s="1"/>
+      <c r="ALL16" s="1"/>
+      <c r="ALM16" s="1"/>
+      <c r="ALN16" s="1"/>
+      <c r="ALO16" s="1"/>
+      <c r="ALP16" s="1"/>
+      <c r="ALQ16" s="1"/>
+      <c r="ALR16" s="1"/>
+      <c r="ALS16" s="1"/>
+      <c r="ALT16" s="1"/>
+      <c r="ALU16" s="1"/>
+      <c r="ALV16" s="1"/>
+      <c r="ALW16" s="1"/>
+      <c r="ALX16" s="1"/>
+      <c r="ALY16" s="1"/>
+      <c r="ALZ16" s="1"/>
+      <c r="AMA16" s="1"/>
+      <c r="AMB16" s="1"/>
+      <c r="AMC16" s="1"/>
+      <c r="AMD16" s="1"/>
+      <c r="AME16" s="1"/>
+      <c r="AMF16" s="1"/>
+      <c r="AMG16" s="1"/>
+      <c r="AMH16" s="1"/>
+      <c r="AMI16" s="1"/>
+      <c r="AMJ16" s="1"/>
+    </row>
+    <row r="17" s="13" customFormat="true" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="12"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12"/>
+      <c r="ALK17" s="1"/>
+      <c r="ALL17" s="1"/>
+      <c r="ALM17" s="1"/>
+      <c r="ALN17" s="1"/>
+      <c r="ALO17" s="1"/>
+      <c r="ALP17" s="1"/>
+      <c r="ALQ17" s="1"/>
+      <c r="ALR17" s="1"/>
+      <c r="ALS17" s="1"/>
+      <c r="ALT17" s="1"/>
+      <c r="ALU17" s="1"/>
+      <c r="ALV17" s="1"/>
+      <c r="ALW17" s="1"/>
+      <c r="ALX17" s="1"/>
+      <c r="ALY17" s="1"/>
+      <c r="ALZ17" s="1"/>
+      <c r="AMA17" s="1"/>
+      <c r="AMB17" s="1"/>
+      <c r="AMC17" s="1"/>
+      <c r="AMD17" s="1"/>
+      <c r="AME17" s="1"/>
+      <c r="AMF17" s="1"/>
+      <c r="AMG17" s="1"/>
+      <c r="AMH17" s="1"/>
+      <c r="AMI17" s="1"/>
+      <c r="AMJ17" s="1"/>
+    </row>
+    <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14"/>
+      <c r="L18" s="14"/>
+      <c r="M18" s="14"/>
+      <c r="N18" s="14"/>
+    </row>
+    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="12"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="12"/>
+      <c r="M19" s="12"/>
+      <c r="N19" s="12"/>
+    </row>
+    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="14"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="14"/>
+      <c r="K20" s="14"/>
+      <c r="L20" s="14"/>
+      <c r="M20" s="14"/>
+      <c r="N20" s="14"/>
+    </row>
+    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="12"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
+      <c r="L21" s="12"/>
+      <c r="M21" s="12"/>
+      <c r="N21" s="12"/>
+    </row>
+    <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="14"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="14"/>
+      <c r="L22" s="14"/>
+      <c r="M22" s="14"/>
+      <c r="N22" s="14"/>
+    </row>
+    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="12"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="12"/>
+      <c r="M23" s="12"/>
+      <c r="N23" s="12"/>
+    </row>
+    <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="14"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="14"/>
+      <c r="H24" s="14"/>
+      <c r="I24" s="14"/>
+      <c r="J24" s="14"/>
+      <c r="K24" s="14"/>
+      <c r="L24" s="14"/>
+      <c r="M24" s="14"/>
+      <c r="N24" s="14"/>
+    </row>
+    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="12"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="12"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="12"/>
+      <c r="M25" s="12"/>
+      <c r="N25" s="12"/>
+    </row>
+    <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="14"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="14"/>
+      <c r="I26" s="14"/>
+      <c r="J26" s="14"/>
+      <c r="K26" s="14"/>
+      <c r="L26" s="14"/>
+      <c r="M26" s="14"/>
+      <c r="N26" s="14"/>
+    </row>
+    <row r="27" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="12"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="12"/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="12"/>
+      <c r="L27" s="12"/>
+      <c r="M27" s="12"/>
+      <c r="N27" s="12"/>
+    </row>
+    <row r="28" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="14"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="14"/>
+      <c r="H28" s="14"/>
+      <c r="I28" s="14"/>
+      <c r="J28" s="14"/>
+      <c r="K28" s="14"/>
+      <c r="L28" s="14"/>
+      <c r="M28" s="14"/>
+      <c r="N28" s="14"/>
+    </row>
+    <row r="29" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="12"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+      <c r="I29" s="12"/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="12"/>
+      <c r="L29" s="12"/>
+      <c r="M29" s="12"/>
+      <c r="N29" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="14"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
+      <c r="I30" s="14"/>
+      <c r="J30" s="14"/>
+      <c r="K30" s="14"/>
+      <c r="L30" s="14"/>
+      <c r="M30" s="14"/>
+      <c r="N30" s="14"/>
+    </row>
+    <row r="31" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="12"/>
+      <c r="B31" s="12"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="12"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="12"/>
+      <c r="I31" s="12"/>
+      <c r="J31" s="12"/>
+      <c r="K31" s="12"/>
+      <c r="L31" s="12"/>
+      <c r="M31" s="12"/>
+      <c r="N31" s="12"/>
+    </row>
+    <row r="32" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="14"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="14"/>
+      <c r="I32" s="14"/>
+      <c r="J32" s="14"/>
+      <c r="K32" s="14"/>
+      <c r="L32" s="14"/>
+      <c r="M32" s="14"/>
+      <c r="N32" s="14"/>
+    </row>
+    <row r="33" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="12"/>
+      <c r="B33" s="12"/>
+      <c r="C33" s="12"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="12"/>
+      <c r="F33" s="12"/>
+      <c r="G33" s="12"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="12"/>
+      <c r="J33" s="12"/>
+      <c r="K33" s="12"/>
+      <c r="L33" s="12"/>
+      <c r="M33" s="12"/>
+      <c r="N33" s="12"/>
+    </row>
+    <row r="34" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="14"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
+      <c r="I34" s="14"/>
+      <c r="J34" s="14"/>
+      <c r="K34" s="14"/>
+      <c r="L34" s="14"/>
+      <c r="M34" s="14"/>
+      <c r="N34" s="14"/>
+    </row>
+    <row r="35" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="12"/>
+      <c r="B35" s="12"/>
+      <c r="C35" s="12"/>
+      <c r="D35" s="12"/>
+      <c r="E35" s="12"/>
+      <c r="F35" s="12"/>
+      <c r="G35" s="12"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="12"/>
+      <c r="J35" s="12"/>
+      <c r="K35" s="12"/>
+      <c r="L35" s="12"/>
+      <c r="M35" s="12"/>
+      <c r="N35" s="12"/>
+    </row>
+    <row r="36" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="14"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="14"/>
+      <c r="H36" s="14"/>
+      <c r="I36" s="14"/>
+      <c r="J36" s="14"/>
+      <c r="K36" s="14"/>
+      <c r="L36" s="14"/>
+      <c r="M36" s="14"/>
+      <c r="N36" s="14"/>
+    </row>
+    <row r="37" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="12"/>
+      <c r="B37" s="12"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="12"/>
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
+      <c r="I37" s="12"/>
+      <c r="J37" s="12"/>
+      <c r="K37" s="12"/>
+      <c r="L37" s="12"/>
+      <c r="M37" s="12"/>
+      <c r="N37" s="12"/>
+    </row>
+    <row r="38" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="14"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="14"/>
+      <c r="H38" s="14"/>
+      <c r="I38" s="14"/>
+      <c r="J38" s="14"/>
+      <c r="K38" s="14"/>
+      <c r="L38" s="14"/>
+      <c r="M38" s="14"/>
+      <c r="N38" s="14"/>
+    </row>
+    <row r="39" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="12"/>
+      <c r="B39" s="12"/>
+      <c r="C39" s="12"/>
+      <c r="D39" s="12"/>
+      <c r="E39" s="12"/>
+      <c r="F39" s="12"/>
+      <c r="G39" s="12"/>
+      <c r="H39" s="12"/>
+      <c r="I39" s="12"/>
+      <c r="J39" s="12"/>
+      <c r="K39" s="12"/>
+      <c r="L39" s="12"/>
+      <c r="M39" s="12"/>
+      <c r="N39" s="12"/>
+    </row>
+    <row r="40" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="14"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="14"/>
+      <c r="G40" s="14"/>
+      <c r="H40" s="14"/>
+      <c r="I40" s="14"/>
+      <c r="J40" s="14"/>
+      <c r="K40" s="14"/>
+      <c r="L40" s="14"/>
+      <c r="M40" s="14"/>
+      <c r="N40" s="14"/>
+    </row>
+    <row r="41" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="12"/>
+      <c r="B41" s="12"/>
+      <c r="C41" s="12"/>
+      <c r="D41" s="12"/>
+      <c r="E41" s="12"/>
+      <c r="F41" s="12"/>
+      <c r="G41" s="12"/>
+      <c r="H41" s="12"/>
+      <c r="I41" s="12"/>
+      <c r="J41" s="12"/>
+      <c r="K41" s="12"/>
+      <c r="L41" s="12"/>
+      <c r="M41" s="12"/>
+      <c r="N41" s="12"/>
+    </row>
+    <row r="42" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="14"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="14"/>
+      <c r="G42" s="14"/>
+      <c r="H42" s="14"/>
+      <c r="I42" s="14"/>
+      <c r="J42" s="14"/>
+      <c r="K42" s="14"/>
+      <c r="L42" s="14"/>
+      <c r="M42" s="14"/>
+      <c r="N42" s="14"/>
+    </row>
+    <row r="43" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="12"/>
+      <c r="B43" s="12"/>
+      <c r="C43" s="12"/>
+      <c r="D43" s="12"/>
+      <c r="E43" s="12"/>
+      <c r="F43" s="12"/>
+      <c r="G43" s="12"/>
+      <c r="H43" s="12"/>
+      <c r="I43" s="12"/>
+      <c r="J43" s="12"/>
+      <c r="K43" s="12"/>
+      <c r="L43" s="12"/>
+      <c r="M43" s="12"/>
+      <c r="N43" s="12"/>
+    </row>
+    <row r="44" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="14"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="14"/>
+      <c r="F44" s="14"/>
+      <c r="G44" s="14"/>
+      <c r="H44" s="14"/>
+      <c r="I44" s="14"/>
+      <c r="J44" s="14"/>
+      <c r="K44" s="14"/>
+      <c r="L44" s="14"/>
+      <c r="M44" s="14"/>
+      <c r="N44" s="14"/>
+    </row>
+    <row r="45" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="15"/>
+      <c r="B45" s="15"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="15"/>
+      <c r="F45" s="15"/>
+      <c r="G45" s="15"/>
+      <c r="H45" s="15"/>
+      <c r="I45" s="15"/>
+      <c r="J45" s="15"/>
+      <c r="K45" s="15"/>
+      <c r="L45" s="15"/>
+      <c r="M45" s="15"/>
+      <c r="N45" s="15"/>
+    </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -5655,13 +6183,6 @@
     <row r="999" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1000" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="N1:O1"/>
-  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -5677,1580 +6198,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AMJ1000"/>
-  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="3" style="1" width="10.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="9.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="12.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="999" style="1" width="11.52"/>
-  </cols>
-  <sheetData>
-    <row r="1" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="N1" s="11"/>
-      <c r="O1" s="11"/>
-      <c r="ALK1" s="1"/>
-      <c r="ALL1" s="1"/>
-      <c r="ALM1" s="1"/>
-      <c r="ALN1" s="1"/>
-      <c r="ALO1" s="1"/>
-      <c r="ALP1" s="1"/>
-      <c r="ALQ1" s="1"/>
-      <c r="ALR1" s="1"/>
-      <c r="ALS1" s="1"/>
-      <c r="ALT1" s="1"/>
-      <c r="ALU1" s="1"/>
-      <c r="ALV1" s="1"/>
-      <c r="ALW1" s="1"/>
-      <c r="ALX1" s="1"/>
-      <c r="ALY1" s="1"/>
-      <c r="ALZ1" s="1"/>
-      <c r="AMA1" s="1"/>
-      <c r="AMB1" s="1"/>
-      <c r="AMC1" s="1"/>
-      <c r="AMD1" s="1"/>
-      <c r="AME1" s="1"/>
-      <c r="AMF1" s="1"/>
-      <c r="AMG1" s="1"/>
-      <c r="AMH1" s="1"/>
-      <c r="AMI1" s="1"/>
-      <c r="AMJ1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="16" s="10" customFormat="true" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="12"/>
-      <c r="J16" s="12"/>
-      <c r="K16" s="12"/>
-      <c r="L16" s="12"/>
-      <c r="M16" s="12"/>
-      <c r="N16" s="12"/>
-      <c r="ALK16" s="1"/>
-      <c r="ALL16" s="1"/>
-      <c r="ALM16" s="1"/>
-      <c r="ALN16" s="1"/>
-      <c r="ALO16" s="1"/>
-      <c r="ALP16" s="1"/>
-      <c r="ALQ16" s="1"/>
-      <c r="ALR16" s="1"/>
-      <c r="ALS16" s="1"/>
-      <c r="ALT16" s="1"/>
-      <c r="ALU16" s="1"/>
-      <c r="ALV16" s="1"/>
-      <c r="ALW16" s="1"/>
-      <c r="ALX16" s="1"/>
-      <c r="ALY16" s="1"/>
-      <c r="ALZ16" s="1"/>
-      <c r="AMA16" s="1"/>
-      <c r="AMB16" s="1"/>
-      <c r="AMC16" s="1"/>
-      <c r="AMD16" s="1"/>
-      <c r="AME16" s="1"/>
-      <c r="AMF16" s="1"/>
-      <c r="AMG16" s="1"/>
-      <c r="AMH16" s="1"/>
-      <c r="AMI16" s="1"/>
-      <c r="AMJ16" s="1"/>
-    </row>
-    <row r="17" s="14" customFormat="true" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13"/>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="13"/>
-      <c r="J17" s="13"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="13"/>
-      <c r="M17" s="13"/>
-      <c r="N17" s="13"/>
-      <c r="ALK17" s="1"/>
-      <c r="ALL17" s="1"/>
-      <c r="ALM17" s="1"/>
-      <c r="ALN17" s="1"/>
-      <c r="ALO17" s="1"/>
-      <c r="ALP17" s="1"/>
-      <c r="ALQ17" s="1"/>
-      <c r="ALR17" s="1"/>
-      <c r="ALS17" s="1"/>
-      <c r="ALT17" s="1"/>
-      <c r="ALU17" s="1"/>
-      <c r="ALV17" s="1"/>
-      <c r="ALW17" s="1"/>
-      <c r="ALX17" s="1"/>
-      <c r="ALY17" s="1"/>
-      <c r="ALZ17" s="1"/>
-      <c r="AMA17" s="1"/>
-      <c r="AMB17" s="1"/>
-      <c r="AMC17" s="1"/>
-      <c r="AMD17" s="1"/>
-      <c r="AME17" s="1"/>
-      <c r="AMF17" s="1"/>
-      <c r="AMG17" s="1"/>
-      <c r="AMH17" s="1"/>
-      <c r="AMI17" s="1"/>
-      <c r="AMJ17" s="1"/>
-    </row>
-    <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="15"/>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="15"/>
-      <c r="M18" s="15"/>
-      <c r="N18" s="15"/>
-    </row>
-    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="13"/>
-      <c r="I19" s="13"/>
-      <c r="J19" s="13"/>
-      <c r="K19" s="13"/>
-      <c r="L19" s="13"/>
-      <c r="M19" s="13"/>
-      <c r="N19" s="13"/>
-    </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15"/>
-      <c r="B20" s="15"/>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15"/>
-      <c r="G20" s="15"/>
-      <c r="H20" s="15"/>
-      <c r="I20" s="15"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="15"/>
-      <c r="L20" s="15"/>
-      <c r="M20" s="15"/>
-      <c r="N20" s="15"/>
-    </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="13"/>
-      <c r="J21" s="13"/>
-      <c r="K21" s="13"/>
-      <c r="L21" s="13"/>
-      <c r="M21" s="13"/>
-      <c r="N21" s="13"/>
-    </row>
-    <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15"/>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="15"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="15"/>
-      <c r="L22" s="15"/>
-      <c r="M22" s="15"/>
-      <c r="N22" s="15"/>
-    </row>
-    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="13"/>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="13"/>
-      <c r="J23" s="13"/>
-      <c r="K23" s="13"/>
-      <c r="L23" s="13"/>
-      <c r="M23" s="13"/>
-      <c r="N23" s="13"/>
-    </row>
-    <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15"/>
-      <c r="B24" s="15"/>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="15"/>
-      <c r="I24" s="15"/>
-      <c r="J24" s="15"/>
-      <c r="K24" s="15"/>
-      <c r="L24" s="15"/>
-      <c r="M24" s="15"/>
-      <c r="N24" s="15"/>
-    </row>
-    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="13"/>
-      <c r="H25" s="13"/>
-      <c r="I25" s="13"/>
-      <c r="J25" s="13"/>
-      <c r="K25" s="13"/>
-      <c r="L25" s="13"/>
-      <c r="M25" s="13"/>
-      <c r="N25" s="13"/>
-    </row>
-    <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="15"/>
-      <c r="B26" s="15"/>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="15"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="15"/>
-      <c r="I26" s="15"/>
-      <c r="J26" s="15"/>
-      <c r="K26" s="15"/>
-      <c r="L26" s="15"/>
-      <c r="M26" s="15"/>
-      <c r="N26" s="15"/>
-    </row>
-    <row r="27" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="13"/>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="13"/>
-      <c r="H27" s="13"/>
-      <c r="I27" s="13"/>
-      <c r="J27" s="13"/>
-      <c r="K27" s="13"/>
-      <c r="L27" s="13"/>
-      <c r="M27" s="13"/>
-      <c r="N27" s="13"/>
-    </row>
-    <row r="28" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15"/>
-      <c r="B28" s="15"/>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="15"/>
-      <c r="G28" s="15"/>
-      <c r="H28" s="15"/>
-      <c r="I28" s="15"/>
-      <c r="J28" s="15"/>
-      <c r="K28" s="15"/>
-      <c r="L28" s="15"/>
-      <c r="M28" s="15"/>
-      <c r="N28" s="15"/>
-    </row>
-    <row r="29" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="13"/>
-      <c r="B29" s="13"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="13"/>
-      <c r="H29" s="13"/>
-      <c r="I29" s="13"/>
-      <c r="J29" s="13"/>
-      <c r="K29" s="13"/>
-      <c r="L29" s="13"/>
-      <c r="M29" s="13"/>
-      <c r="N29" s="13"/>
-    </row>
-    <row r="30" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15"/>
-      <c r="B30" s="15"/>
-      <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="15"/>
-      <c r="F30" s="15"/>
-      <c r="G30" s="15"/>
-      <c r="H30" s="15"/>
-      <c r="I30" s="15"/>
-      <c r="J30" s="15"/>
-      <c r="K30" s="15"/>
-      <c r="L30" s="15"/>
-      <c r="M30" s="15"/>
-      <c r="N30" s="15"/>
-    </row>
-    <row r="31" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="13"/>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="13"/>
-      <c r="H31" s="13"/>
-      <c r="I31" s="13"/>
-      <c r="J31" s="13"/>
-      <c r="K31" s="13"/>
-      <c r="L31" s="13"/>
-      <c r="M31" s="13"/>
-      <c r="N31" s="13"/>
-    </row>
-    <row r="32" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="15"/>
-      <c r="B32" s="15"/>
-      <c r="C32" s="15"/>
-      <c r="D32" s="15"/>
-      <c r="E32" s="15"/>
-      <c r="F32" s="15"/>
-      <c r="G32" s="15"/>
-      <c r="H32" s="15"/>
-      <c r="I32" s="15"/>
-      <c r="J32" s="15"/>
-      <c r="K32" s="15"/>
-      <c r="L32" s="15"/>
-      <c r="M32" s="15"/>
-      <c r="N32" s="15"/>
-    </row>
-    <row r="33" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="13"/>
-      <c r="B33" s="13"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="13"/>
-      <c r="I33" s="13"/>
-      <c r="J33" s="13"/>
-      <c r="K33" s="13"/>
-      <c r="L33" s="13"/>
-      <c r="M33" s="13"/>
-      <c r="N33" s="13"/>
-    </row>
-    <row r="34" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="15"/>
-      <c r="B34" s="15"/>
-      <c r="C34" s="15"/>
-      <c r="D34" s="15"/>
-      <c r="E34" s="15"/>
-      <c r="F34" s="15"/>
-      <c r="G34" s="15"/>
-      <c r="H34" s="15"/>
-      <c r="I34" s="15"/>
-      <c r="J34" s="15"/>
-      <c r="K34" s="15"/>
-      <c r="L34" s="15"/>
-      <c r="M34" s="15"/>
-      <c r="N34" s="15"/>
-    </row>
-    <row r="35" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="13"/>
-      <c r="B35" s="13"/>
-      <c r="C35" s="13"/>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="13"/>
-      <c r="H35" s="13"/>
-      <c r="I35" s="13"/>
-      <c r="J35" s="13"/>
-      <c r="K35" s="13"/>
-      <c r="L35" s="13"/>
-      <c r="M35" s="13"/>
-      <c r="N35" s="13"/>
-    </row>
-    <row r="36" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="15"/>
-      <c r="B36" s="15"/>
-      <c r="C36" s="15"/>
-      <c r="D36" s="15"/>
-      <c r="E36" s="15"/>
-      <c r="F36" s="15"/>
-      <c r="G36" s="15"/>
-      <c r="H36" s="15"/>
-      <c r="I36" s="15"/>
-      <c r="J36" s="15"/>
-      <c r="K36" s="15"/>
-      <c r="L36" s="15"/>
-      <c r="M36" s="15"/>
-      <c r="N36" s="15"/>
-    </row>
-    <row r="37" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="13"/>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="13"/>
-      <c r="G37" s="13"/>
-      <c r="H37" s="13"/>
-      <c r="I37" s="13"/>
-      <c r="J37" s="13"/>
-      <c r="K37" s="13"/>
-      <c r="L37" s="13"/>
-      <c r="M37" s="13"/>
-      <c r="N37" s="13"/>
-    </row>
-    <row r="38" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="15"/>
-      <c r="B38" s="15"/>
-      <c r="C38" s="15"/>
-      <c r="D38" s="15"/>
-      <c r="E38" s="15"/>
-      <c r="F38" s="15"/>
-      <c r="G38" s="15"/>
-      <c r="H38" s="15"/>
-      <c r="I38" s="15"/>
-      <c r="J38" s="15"/>
-      <c r="K38" s="15"/>
-      <c r="L38" s="15"/>
-      <c r="M38" s="15"/>
-      <c r="N38" s="15"/>
-    </row>
-    <row r="39" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="13"/>
-      <c r="B39" s="13"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="13"/>
-      <c r="H39" s="13"/>
-      <c r="I39" s="13"/>
-      <c r="J39" s="13"/>
-      <c r="K39" s="13"/>
-      <c r="L39" s="13"/>
-      <c r="M39" s="13"/>
-      <c r="N39" s="13"/>
-    </row>
-    <row r="40" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="15"/>
-      <c r="B40" s="15"/>
-      <c r="C40" s="15"/>
-      <c r="D40" s="15"/>
-      <c r="E40" s="15"/>
-      <c r="F40" s="15"/>
-      <c r="G40" s="15"/>
-      <c r="H40" s="15"/>
-      <c r="I40" s="15"/>
-      <c r="J40" s="15"/>
-      <c r="K40" s="15"/>
-      <c r="L40" s="15"/>
-      <c r="M40" s="15"/>
-      <c r="N40" s="15"/>
-    </row>
-    <row r="41" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="13"/>
-      <c r="B41" s="13"/>
-      <c r="C41" s="13"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="13"/>
-      <c r="F41" s="13"/>
-      <c r="G41" s="13"/>
-      <c r="H41" s="13"/>
-      <c r="I41" s="13"/>
-      <c r="J41" s="13"/>
-      <c r="K41" s="13"/>
-      <c r="L41" s="13"/>
-      <c r="M41" s="13"/>
-      <c r="N41" s="13"/>
-    </row>
-    <row r="42" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="15"/>
-      <c r="B42" s="15"/>
-      <c r="C42" s="15"/>
-      <c r="D42" s="15"/>
-      <c r="E42" s="15"/>
-      <c r="F42" s="15"/>
-      <c r="G42" s="15"/>
-      <c r="H42" s="15"/>
-      <c r="I42" s="15"/>
-      <c r="J42" s="15"/>
-      <c r="K42" s="15"/>
-      <c r="L42" s="15"/>
-      <c r="M42" s="15"/>
-      <c r="N42" s="15"/>
-    </row>
-    <row r="43" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="13"/>
-      <c r="B43" s="13"/>
-      <c r="C43" s="13"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
-      <c r="F43" s="13"/>
-      <c r="G43" s="13"/>
-      <c r="H43" s="13"/>
-      <c r="I43" s="13"/>
-      <c r="J43" s="13"/>
-      <c r="K43" s="13"/>
-      <c r="L43" s="13"/>
-      <c r="M43" s="13"/>
-      <c r="N43" s="13"/>
-    </row>
-    <row r="44" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="15"/>
-      <c r="B44" s="15"/>
-      <c r="C44" s="15"/>
-      <c r="D44" s="15"/>
-      <c r="E44" s="15"/>
-      <c r="F44" s="15"/>
-      <c r="G44" s="15"/>
-      <c r="H44" s="15"/>
-      <c r="I44" s="15"/>
-      <c r="J44" s="15"/>
-      <c r="K44" s="15"/>
-      <c r="L44" s="15"/>
-      <c r="M44" s="15"/>
-      <c r="N44" s="15"/>
-    </row>
-    <row r="45" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="16"/>
-      <c r="B45" s="16"/>
-      <c r="C45" s="16"/>
-      <c r="D45" s="16"/>
-      <c r="E45" s="16"/>
-      <c r="F45" s="16"/>
-      <c r="G45" s="16"/>
-      <c r="H45" s="16"/>
-      <c r="I45" s="16"/>
-      <c r="J45" s="16"/>
-      <c r="K45" s="16"/>
-      <c r="L45" s="16"/>
-      <c r="M45" s="16"/>
-      <c r="N45" s="16"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="81" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="92" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="93" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="94" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="95" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="96" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="97" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="98" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="99" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="100" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="101" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="102" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="103" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="104" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="105" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="106" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="107" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="108" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="109" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="110" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="111" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="112" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="113" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="114" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="115" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="116" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="117" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="118" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="119" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="120" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="121" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="122" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="123" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="124" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="125" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="126" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="127" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="128" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="129" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="130" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="131" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="132" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="133" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="134" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="135" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="136" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="137" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="138" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="139" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="140" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="141" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="142" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="143" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="144" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="145" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="146" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="147" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="148" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="149" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="150" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="151" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="152" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="153" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="154" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="155" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="156" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="157" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="158" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="159" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="160" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="161" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="162" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="163" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="164" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="165" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="166" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="167" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="168" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="169" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="170" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="171" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="172" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="173" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="174" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="175" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="176" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="177" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="178" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="179" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="180" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="181" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="182" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="183" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="184" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="185" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="186" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="187" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="188" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="189" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="190" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="191" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="192" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="193" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="194" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="195" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="196" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="197" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="198" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="199" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="200" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="201" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="202" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="203" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="204" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="205" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="206" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="207" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="208" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="209" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="210" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="211" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="212" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="213" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="214" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="215" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="216" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="217" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="218" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="219" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="220" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="221" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="222" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="223" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="224" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="225" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="226" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="227" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="228" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="229" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="230" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="231" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="232" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="233" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="234" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="235" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="236" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="237" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="238" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="239" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="240" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="241" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="242" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="243" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="244" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="245" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="246" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="247" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="248" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="249" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="250" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="251" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="252" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="253" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="254" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="255" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="256" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="257" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="258" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="259" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="260" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="261" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="262" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="263" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="264" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="265" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="266" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="267" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="268" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="269" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="270" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="271" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="272" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="273" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="274" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="275" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="276" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="277" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="278" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="279" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="280" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="281" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="282" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="283" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="284" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="285" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="286" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="287" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="288" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="289" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="290" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="291" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="292" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="293" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="294" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="295" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="296" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="297" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="298" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="299" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="300" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="301" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="302" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="303" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="304" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="305" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="306" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="307" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="308" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="309" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="310" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="311" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="312" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="313" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="314" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="315" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="316" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="317" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="318" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="319" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="320" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="321" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="322" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="323" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="324" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="325" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="326" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="327" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="328" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="329" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="330" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="331" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="332" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="333" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="334" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="335" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="336" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="337" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="338" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="339" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="340" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="341" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="342" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="343" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="344" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="345" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="346" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="347" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="348" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="349" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="350" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="351" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="352" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="353" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="354" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="355" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="356" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="357" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="358" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="359" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="360" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="361" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="362" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="363" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="364" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="365" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="366" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="367" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="368" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="369" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="370" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="371" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="372" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="373" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="374" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="375" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="376" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="377" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="378" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="379" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="380" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="381" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="382" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="383" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="384" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="385" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="386" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="387" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="388" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="389" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="390" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="391" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="392" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="393" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="394" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="395" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="396" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="397" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="398" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="399" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="400" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="401" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="402" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="403" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="404" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="405" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="406" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="407" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="408" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="409" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="410" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="411" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="412" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="413" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="414" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="415" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="416" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="417" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="418" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="419" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="420" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="421" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="422" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="423" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="424" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="425" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="426" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="427" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="428" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="429" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="430" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="431" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="432" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="433" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="434" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="435" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="436" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="437" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="438" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="439" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="440" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="441" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="442" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="443" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="444" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="445" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="446" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="447" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="448" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="449" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="450" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="451" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="452" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="453" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="454" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="455" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="456" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="457" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="458" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="459" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="460" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="461" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="462" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="463" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="464" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="465" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="466" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="467" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="468" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="469" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="470" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="471" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="472" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="473" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="474" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="475" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="476" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="477" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="478" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="479" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="480" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="481" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="482" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="483" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="484" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="485" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="486" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="487" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="488" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="489" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="490" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="491" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="492" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="493" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="494" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="495" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="496" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="497" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="498" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="499" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="500" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="501" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="502" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="503" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="504" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="505" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="506" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="507" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="508" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="509" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="510" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="511" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="512" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="513" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="514" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="515" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="516" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="517" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="518" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="519" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="520" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="521" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="522" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="523" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="524" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="525" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="526" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="527" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="528" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="529" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="530" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="531" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="532" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="533" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="534" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="535" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="536" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="537" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="538" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="539" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="540" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="541" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="542" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="543" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="544" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="545" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="546" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="547" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="548" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="549" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="550" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="551" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="552" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="553" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="554" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="555" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="556" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="557" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="558" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="559" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="560" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="561" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="562" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="563" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="564" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="565" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="566" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="567" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="568" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="569" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="570" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="571" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="572" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="573" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="574" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="575" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="576" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="577" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="578" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="579" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="580" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="581" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="582" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="583" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="584" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="585" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="586" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="587" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="588" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="589" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="590" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="591" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="592" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="593" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="594" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="595" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="596" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="597" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="598" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="599" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="600" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="601" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="602" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="603" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="604" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="605" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="606" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="607" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="608" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="609" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="610" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="611" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="612" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="613" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="614" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="615" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="616" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="617" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="618" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="619" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="620" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="621" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="622" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="623" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="624" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="625" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="626" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="627" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="628" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="629" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="630" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="631" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="632" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="633" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="634" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="635" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="636" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="637" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="638" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="639" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="640" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="641" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="642" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="643" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="644" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="645" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="646" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="647" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="648" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="649" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="650" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="651" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="652" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="653" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="654" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="655" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="656" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="657" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="658" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="659" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="660" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="661" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="662" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="663" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="664" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="665" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="666" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="667" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="668" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="669" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="670" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="671" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="672" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="673" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="674" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="675" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="676" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="677" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="678" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="679" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="680" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="681" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="682" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="683" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="684" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="685" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="686" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="687" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="688" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="689" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="690" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="691" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="692" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="693" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="694" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="695" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="696" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="697" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="698" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="699" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="700" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="701" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="702" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="703" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="704" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="705" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="706" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="707" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="708" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="709" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="710" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="711" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="712" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="713" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="714" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="715" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="716" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="717" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="718" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="719" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="720" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="721" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="722" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="723" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="724" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="725" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="726" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="727" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="728" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="729" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="730" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="731" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="732" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="733" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="734" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="735" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="736" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="737" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="738" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="739" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="740" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="741" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="742" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="743" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="744" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="745" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="746" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="747" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="748" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="749" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="750" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="751" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="752" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="753" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="754" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="755" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="756" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="757" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="758" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="759" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="760" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="761" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="762" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="763" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="764" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="765" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="766" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="767" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="768" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="769" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="770" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="771" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="772" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="773" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="774" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="775" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="776" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="777" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="778" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="779" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="780" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="781" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="782" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="783" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="784" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="785" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="786" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="787" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="788" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="789" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="790" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="791" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="792" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="793" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="794" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="795" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="796" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="797" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="798" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="799" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="800" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="801" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="802" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="803" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="804" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="805" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="806" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="807" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="808" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="809" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="810" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="811" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="812" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="813" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="814" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="815" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="816" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="817" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="818" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="819" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="820" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="821" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="822" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="823" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="824" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="825" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="826" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="827" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="828" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="829" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="830" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="831" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="832" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="833" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="834" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="835" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="836" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="837" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="838" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="839" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="840" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="841" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="842" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="843" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="844" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="845" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="846" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="847" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="848" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="849" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="850" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="851" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="852" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="853" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="854" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="855" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="856" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="857" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="858" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="859" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="860" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="861" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="862" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="863" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="864" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="865" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="866" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="867" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="868" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="869" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="870" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="871" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="872" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="873" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="874" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="875" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="876" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="877" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="878" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="879" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="880" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="881" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="882" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="883" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="884" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="885" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="886" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="887" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="888" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="889" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="890" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="891" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="892" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="893" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="894" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="895" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="896" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="897" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="898" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="899" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="900" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="901" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="902" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="903" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="904" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="905" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="906" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="907" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="908" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="909" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="910" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="911" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="912" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="913" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="914" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="915" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="916" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="917" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="918" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="919" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="920" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="921" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="922" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="923" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="924" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="925" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="926" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="927" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="928" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="929" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="930" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="931" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="932" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="933" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="934" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="935" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="936" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="937" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="938" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="939" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="940" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="941" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="942" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="943" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="944" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="945" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="946" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="947" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="948" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="949" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="950" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="951" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="952" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="953" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="954" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="955" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="956" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="957" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="958" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="959" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="960" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="961" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="962" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="963" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="964" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="965" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="966" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="967" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="968" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="969" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="970" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="971" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="972" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="973" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="974" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="975" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="976" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="977" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="978" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="979" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="980" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="981" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="982" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="983" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="984" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="985" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="986" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="987" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="988" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="989" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="990" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="991" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="992" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="993" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="994" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="995" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="996" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="997" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="998" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="999" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1000" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="N1:O1"/>
-  </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="13.2734375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="13.30859375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.5"/>
@@ -8275,13 +7224,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C39"/>
-  <sheetFormatPr defaultColWidth="11.94140625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.9765625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="9" width="11.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22.62"/>
@@ -8481,13 +7430,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:T86"/>
-  <sheetFormatPr defaultColWidth="11.94140625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.9765625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="11.69"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25.52"/>
@@ -8502,40 +7451,40 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
-      <c r="P1" s="18"/>
-      <c r="Q1" s="18"/>
-      <c r="R1" s="19"/>
-      <c r="S1" s="19"/>
-      <c r="T1" s="20"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17"/>
+      <c r="Q1" s="17"/>
+      <c r="R1" s="18"/>
+      <c r="S1" s="18"/>
+      <c r="T1" s="19"/>
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17"/>
-      <c r="B2" s="21" t="n">
+      <c r="A2" s="16"/>
+      <c r="B2" s="20" t="n">
         <f aca="false">VLOOKUP("a1", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C2" s="21" t="n">
+      <c r="C2" s="20" t="n">
         <f aca="false">VLOOKUP("a1", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D2" s="22"/>
+      <c r="D2" s="21"/>
       <c r="E2" s="22"/>
       <c r="F2" s="22"/>
       <c r="G2" s="5"/>
@@ -8548,7 +7497,7 @@
       <c r="T2" s="23"/>
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="17"/>
+      <c r="A3" s="16"/>
       <c r="B3" s="24" t="n">
         <f aca="false">VLOOKUP("c2", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
@@ -8558,8 +7507,8 @@
         <v>0</v>
       </c>
       <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
       <c r="G3" s="26"/>
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>
@@ -8570,7 +7519,7 @@
       <c r="T3" s="23"/>
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17"/>
+      <c r="A4" s="16"/>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
       <c r="D4" s="6"/>
@@ -8578,16 +7527,16 @@
       <c r="F4" s="6"/>
       <c r="G4" s="27"/>
       <c r="H4" s="28"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="22"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="21"/>
       <c r="L4" s="22"/>
       <c r="M4" s="22"/>
       <c r="N4" s="28"/>
       <c r="T4" s="23"/>
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17"/>
+      <c r="A5" s="16"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="6"/>
@@ -8598,22 +7547,22 @@
       <c r="I5" s="24"/>
       <c r="J5" s="24"/>
       <c r="K5" s="25"/>
-      <c r="L5" s="25"/>
-      <c r="M5" s="25"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="22"/>
       <c r="N5" s="27"/>
       <c r="T5" s="23"/>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17"/>
-      <c r="B6" s="21" t="n">
+      <c r="A6" s="16"/>
+      <c r="B6" s="20" t="n">
         <f aca="false">VLOOKUP("a2", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="20" t="n">
         <f aca="false">VLOOKUP("a2", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D6" s="22"/>
+      <c r="D6" s="21"/>
       <c r="E6" s="22"/>
       <c r="F6" s="22"/>
       <c r="G6" s="29"/>
@@ -8631,7 +7580,7 @@
       <c r="T6" s="30"/>
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17"/>
+      <c r="A7" s="16"/>
       <c r="B7" s="24" t="n">
         <f aca="false">VLOOKUP("c1", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
@@ -8641,8 +7590,8 @@
         <v>0</v>
       </c>
       <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
@@ -8652,23 +7601,23 @@
       <c r="M7" s="6"/>
       <c r="N7" s="27"/>
       <c r="O7" s="28"/>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="22"/>
+      <c r="P7" s="20"/>
+      <c r="Q7" s="20"/>
+      <c r="R7" s="21"/>
       <c r="S7" s="22"/>
       <c r="T7" s="22"/>
     </row>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17"/>
+      <c r="A8" s="16"/>
       <c r="N8" s="27"/>
       <c r="P8" s="24"/>
       <c r="Q8" s="24"/>
       <c r="R8" s="25"/>
-      <c r="S8" s="25"/>
-      <c r="T8" s="25"/>
+      <c r="S8" s="22"/>
+      <c r="T8" s="22"/>
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17"/>
+      <c r="A9" s="16"/>
       <c r="N9" s="27"/>
       <c r="P9" s="5"/>
       <c r="Q9" s="5"/>
@@ -8677,16 +7626,16 @@
       <c r="T9" s="30"/>
     </row>
     <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17"/>
-      <c r="B10" s="21" t="n">
+      <c r="A10" s="16"/>
+      <c r="B10" s="20" t="n">
         <f aca="false">VLOOKUP("b1", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C10" s="20" t="n">
         <f aca="false">VLOOKUP("b1", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="22"/>
+      <c r="D10" s="21"/>
       <c r="E10" s="22"/>
       <c r="F10" s="22"/>
       <c r="G10" s="5"/>
@@ -8698,25 +7647,25 @@
       <c r="M10" s="6"/>
       <c r="N10" s="27"/>
       <c r="O10" s="28"/>
-      <c r="P10" s="21"/>
-      <c r="Q10" s="21"/>
-      <c r="R10" s="22"/>
+      <c r="P10" s="20"/>
+      <c r="Q10" s="20"/>
+      <c r="R10" s="21"/>
       <c r="S10" s="22"/>
       <c r="T10" s="22"/>
     </row>
     <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17"/>
-      <c r="B11" s="21" t="n">
+      <c r="A11" s="16"/>
+      <c r="B11" s="24" t="n">
         <f aca="false">VLOOKUP("d2", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C11" s="21" t="n">
+      <c r="C11" s="24" t="n">
         <f aca="false">VLOOKUP("d2", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
       <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
       <c r="G11" s="26"/>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
@@ -8728,11 +7677,11 @@
       <c r="P11" s="24"/>
       <c r="Q11" s="24"/>
       <c r="R11" s="25"/>
-      <c r="S11" s="25"/>
-      <c r="T11" s="25"/>
+      <c r="S11" s="22"/>
+      <c r="T11" s="22"/>
     </row>
     <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17"/>
+      <c r="A12" s="16"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="6"/>
@@ -8740,9 +7689,9 @@
       <c r="F12" s="6"/>
       <c r="G12" s="27"/>
       <c r="H12" s="28"/>
-      <c r="I12" s="21"/>
-      <c r="J12" s="21"/>
-      <c r="K12" s="22"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="21"/>
       <c r="L12" s="22"/>
       <c r="M12" s="22"/>
       <c r="N12" s="29"/>
@@ -8753,7 +7702,7 @@
       <c r="T12" s="30"/>
     </row>
     <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17"/>
+      <c r="A13" s="16"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="6"/>
@@ -8764,21 +7713,21 @@
       <c r="I13" s="24"/>
       <c r="J13" s="24"/>
       <c r="K13" s="25"/>
-      <c r="L13" s="25"/>
-      <c r="M13" s="25"/>
+      <c r="L13" s="22"/>
+      <c r="M13" s="22"/>
       <c r="T13" s="23"/>
     </row>
     <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17"/>
-      <c r="B14" s="21" t="n">
+      <c r="A14" s="16"/>
+      <c r="B14" s="20" t="n">
         <f aca="false">VLOOKUP("b2", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C14" s="21" t="n">
+      <c r="C14" s="20" t="n">
         <f aca="false">VLOOKUP("b2", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D14" s="22"/>
+      <c r="D14" s="21"/>
       <c r="E14" s="22"/>
       <c r="F14" s="22"/>
       <c r="G14" s="29"/>
@@ -8791,7 +7740,7 @@
       <c r="T14" s="23"/>
     </row>
     <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17"/>
+      <c r="A15" s="16"/>
       <c r="B15" s="24" t="n">
         <f aca="false">VLOOKUP("d1", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
@@ -8801,8 +7750,8 @@
         <v>0</v>
       </c>
       <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
@@ -8813,11 +7762,11 @@
       <c r="T15" s="23"/>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17"/>
+      <c r="A16" s="16"/>
       <c r="T16" s="23"/>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17"/>
+      <c r="A17" s="16"/>
       <c r="B17" s="31"/>
       <c r="C17" s="31"/>
       <c r="D17" s="32"/>
@@ -8839,44 +7788,44 @@
       <c r="T17" s="33"/>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="19"/>
-      <c r="L18" s="19"/>
-      <c r="M18" s="19"/>
-      <c r="N18" s="18"/>
-      <c r="O18" s="18"/>
-      <c r="P18" s="18"/>
-      <c r="Q18" s="18"/>
-      <c r="R18" s="19"/>
-      <c r="S18" s="19"/>
-      <c r="T18" s="20"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="18"/>
+      <c r="L18" s="18"/>
+      <c r="M18" s="18"/>
+      <c r="N18" s="17"/>
+      <c r="O18" s="17"/>
+      <c r="P18" s="17"/>
+      <c r="Q18" s="17"/>
+      <c r="R18" s="18"/>
+      <c r="S18" s="18"/>
+      <c r="T18" s="19"/>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17"/>
+      <c r="A19" s="16"/>
       <c r="T19" s="23"/>
     </row>
     <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17"/>
-      <c r="B20" s="21" t="n">
+      <c r="A20" s="16"/>
+      <c r="B20" s="20" t="n">
         <f aca="false">VLOOKUP("a3", quali_results!$A$1:$C40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C20" s="21" t="n">
+      <c r="C20" s="20" t="n">
         <f aca="false">VLOOKUP("a3", quali_results!$A$1:$C40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D20" s="22"/>
+      <c r="D20" s="21"/>
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
       <c r="G20" s="5"/>
@@ -8889,7 +7838,7 @@
       <c r="T20" s="23"/>
     </row>
     <row r="21" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17"/>
+      <c r="A21" s="16"/>
       <c r="B21" s="24" t="n">
         <f aca="false">VLOOKUP("c4", quali_results!$A$1:$C40,2,0)</f>
         <v>0</v>
@@ -8899,8 +7848,8 @@
         <v>0</v>
       </c>
       <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
       <c r="G21" s="26"/>
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
@@ -8911,7 +7860,7 @@
       <c r="T21" s="23"/>
     </row>
     <row r="22" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17"/>
+      <c r="A22" s="16"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
       <c r="D22" s="6"/>
@@ -8919,16 +7868,16 @@
       <c r="F22" s="6"/>
       <c r="G22" s="27"/>
       <c r="H22" s="28"/>
-      <c r="I22" s="21"/>
-      <c r="J22" s="21"/>
-      <c r="K22" s="22"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="21"/>
       <c r="L22" s="22"/>
       <c r="M22" s="22"/>
       <c r="N22" s="28"/>
       <c r="T22" s="23"/>
     </row>
     <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17"/>
+      <c r="A23" s="16"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
       <c r="D23" s="6"/>
@@ -8939,22 +7888,22 @@
       <c r="I23" s="24"/>
       <c r="J23" s="24"/>
       <c r="K23" s="25"/>
-      <c r="L23" s="25"/>
-      <c r="M23" s="25"/>
+      <c r="L23" s="22"/>
+      <c r="M23" s="22"/>
       <c r="N23" s="27"/>
       <c r="T23" s="23"/>
     </row>
     <row r="24" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17"/>
-      <c r="B24" s="21" t="n">
+      <c r="A24" s="16"/>
+      <c r="B24" s="20" t="n">
         <f aca="false">VLOOKUP("a4", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C24" s="21" t="n">
+      <c r="C24" s="20" t="n">
         <f aca="false">VLOOKUP("a4", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D24" s="22"/>
+      <c r="D24" s="21"/>
       <c r="E24" s="22"/>
       <c r="F24" s="22"/>
       <c r="G24" s="29"/>
@@ -8972,7 +7921,7 @@
       <c r="T24" s="30"/>
     </row>
     <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17"/>
+      <c r="A25" s="16"/>
       <c r="B25" s="24" t="n">
         <f aca="false">VLOOKUP("c3", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
@@ -8982,8 +7931,8 @@
         <v>0</v>
       </c>
       <c r="D25" s="25"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
       <c r="G25" s="5"/>
       <c r="H25" s="5"/>
       <c r="I25" s="5"/>
@@ -8993,23 +7942,23 @@
       <c r="M25" s="6"/>
       <c r="N25" s="27"/>
       <c r="O25" s="28"/>
-      <c r="P25" s="21"/>
-      <c r="Q25" s="21"/>
-      <c r="R25" s="22"/>
+      <c r="P25" s="20"/>
+      <c r="Q25" s="20"/>
+      <c r="R25" s="21"/>
       <c r="S25" s="22"/>
       <c r="T25" s="22"/>
     </row>
     <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17"/>
+      <c r="A26" s="16"/>
       <c r="N26" s="27"/>
       <c r="P26" s="24"/>
       <c r="Q26" s="24"/>
       <c r="R26" s="25"/>
-      <c r="S26" s="25"/>
-      <c r="T26" s="25"/>
+      <c r="S26" s="22"/>
+      <c r="T26" s="22"/>
     </row>
     <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17"/>
+      <c r="A27" s="16"/>
       <c r="N27" s="27"/>
       <c r="P27" s="5"/>
       <c r="Q27" s="5"/>
@@ -9018,16 +7967,16 @@
       <c r="T27" s="30"/>
     </row>
     <row r="28" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17"/>
-      <c r="B28" s="21" t="n">
+      <c r="A28" s="16"/>
+      <c r="B28" s="20" t="n">
         <f aca="false">VLOOKUP("b3", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C28" s="21" t="n">
+      <c r="C28" s="20" t="n">
         <f aca="false">VLOOKUP("b3", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D28" s="22"/>
+      <c r="D28" s="21"/>
       <c r="E28" s="22"/>
       <c r="F28" s="22"/>
       <c r="G28" s="5"/>
@@ -9039,14 +7988,14 @@
       <c r="M28" s="6"/>
       <c r="N28" s="27"/>
       <c r="O28" s="28"/>
-      <c r="P28" s="21"/>
-      <c r="Q28" s="21"/>
-      <c r="R28" s="22"/>
+      <c r="P28" s="20"/>
+      <c r="Q28" s="20"/>
+      <c r="R28" s="21"/>
       <c r="S28" s="22"/>
       <c r="T28" s="22"/>
     </row>
     <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="17"/>
+      <c r="A29" s="16"/>
       <c r="B29" s="24" t="n">
         <f aca="false">VLOOKUP("d4", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
@@ -9056,8 +8005,8 @@
         <v>0</v>
       </c>
       <c r="D29" s="25"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="25"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
       <c r="G29" s="26"/>
       <c r="H29" s="5"/>
       <c r="I29" s="5"/>
@@ -9069,11 +8018,11 @@
       <c r="P29" s="24"/>
       <c r="Q29" s="24"/>
       <c r="R29" s="25"/>
-      <c r="S29" s="25"/>
-      <c r="T29" s="25"/>
+      <c r="S29" s="22"/>
+      <c r="T29" s="22"/>
     </row>
     <row r="30" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="17"/>
+      <c r="A30" s="16"/>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
       <c r="D30" s="6"/>
@@ -9081,9 +8030,9 @@
       <c r="F30" s="6"/>
       <c r="G30" s="27"/>
       <c r="H30" s="28"/>
-      <c r="I30" s="21"/>
-      <c r="J30" s="21"/>
-      <c r="K30" s="22"/>
+      <c r="I30" s="20"/>
+      <c r="J30" s="20"/>
+      <c r="K30" s="21"/>
       <c r="L30" s="22"/>
       <c r="M30" s="22"/>
       <c r="N30" s="29"/>
@@ -9094,7 +8043,7 @@
       <c r="T30" s="30"/>
     </row>
     <row r="31" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="17"/>
+      <c r="A31" s="16"/>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
       <c r="D31" s="6"/>
@@ -9105,21 +8054,21 @@
       <c r="I31" s="24"/>
       <c r="J31" s="24"/>
       <c r="K31" s="25"/>
-      <c r="L31" s="25"/>
-      <c r="M31" s="25"/>
+      <c r="L31" s="22"/>
+      <c r="M31" s="22"/>
       <c r="T31" s="23"/>
     </row>
     <row r="32" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="17"/>
-      <c r="B32" s="21" t="n">
+      <c r="A32" s="16"/>
+      <c r="B32" s="20" t="n">
         <f aca="false">VLOOKUP("b4", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="C32" s="21" t="n">
+      <c r="C32" s="20" t="n">
         <f aca="false">VLOOKUP("b4", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="D32" s="22"/>
+      <c r="D32" s="21"/>
       <c r="E32" s="22"/>
       <c r="F32" s="22"/>
       <c r="G32" s="29"/>
@@ -9132,7 +8081,7 @@
       <c r="T32" s="23"/>
     </row>
     <row r="33" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="17"/>
+      <c r="A33" s="16"/>
       <c r="B33" s="24" t="n">
         <f aca="false">VLOOKUP("d3", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
@@ -9142,8 +8091,8 @@
         <v>0</v>
       </c>
       <c r="D33" s="25"/>
-      <c r="E33" s="25"/>
-      <c r="F33" s="25"/>
+      <c r="E33" s="22"/>
+      <c r="F33" s="22"/>
       <c r="G33" s="5"/>
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
@@ -9154,11 +8103,11 @@
       <c r="T33" s="23"/>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="17"/>
+      <c r="A34" s="16"/>
       <c r="T34" s="23"/>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="17"/>
+      <c r="A35" s="16"/>
       <c r="B35" s="31"/>
       <c r="C35" s="31"/>
       <c r="D35" s="32"/>
@@ -9180,24 +8129,24 @@
       <c r="T35" s="33"/>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="17" t="s">
+      <c r="A36" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="I36" s="18"/>
-      <c r="J36" s="18"/>
-      <c r="K36" s="19"/>
-      <c r="L36" s="19"/>
-      <c r="M36" s="19"/>
-      <c r="N36" s="18"/>
-      <c r="O36" s="18"/>
-      <c r="P36" s="18"/>
-      <c r="Q36" s="18"/>
-      <c r="R36" s="19"/>
-      <c r="S36" s="19"/>
-      <c r="T36" s="20"/>
+      <c r="I36" s="17"/>
+      <c r="J36" s="17"/>
+      <c r="K36" s="18"/>
+      <c r="L36" s="18"/>
+      <c r="M36" s="18"/>
+      <c r="N36" s="17"/>
+      <c r="O36" s="17"/>
+      <c r="P36" s="17"/>
+      <c r="Q36" s="17"/>
+      <c r="R36" s="18"/>
+      <c r="S36" s="18"/>
+      <c r="T36" s="19"/>
     </row>
     <row r="37" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="17"/>
+      <c r="A37" s="16"/>
       <c r="I37" s="5"/>
       <c r="J37" s="5"/>
       <c r="K37" s="6"/>
@@ -9206,7 +8155,7 @@
       <c r="T37" s="23"/>
     </row>
     <row r="38" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="17"/>
+      <c r="A38" s="16"/>
       <c r="I38" s="5"/>
       <c r="J38" s="5"/>
       <c r="K38" s="6"/>
@@ -9215,23 +8164,23 @@
       <c r="T38" s="23"/>
     </row>
     <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="17"/>
-      <c r="I39" s="21" t="n">
+      <c r="A39" s="16"/>
+      <c r="I39" s="20" t="n">
         <f aca="false">VLOOKUP("a5", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="J39" s="21" t="n">
+      <c r="J39" s="20" t="n">
         <f aca="false">VLOOKUP("a5", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="K39" s="22"/>
+      <c r="K39" s="21"/>
       <c r="L39" s="22"/>
       <c r="M39" s="22"/>
       <c r="N39" s="28"/>
       <c r="T39" s="23"/>
     </row>
     <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="17"/>
+      <c r="A40" s="16"/>
       <c r="I40" s="24" t="n">
         <f aca="false">VLOOKUP("c5", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
@@ -9241,13 +8190,13 @@
         <v>0</v>
       </c>
       <c r="K40" s="25"/>
-      <c r="L40" s="25"/>
-      <c r="M40" s="25"/>
+      <c r="L40" s="22"/>
+      <c r="M40" s="22"/>
       <c r="N40" s="27"/>
       <c r="T40" s="23"/>
     </row>
     <row r="41" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="17"/>
+      <c r="A41" s="16"/>
       <c r="I41" s="5"/>
       <c r="J41" s="5"/>
       <c r="K41" s="6"/>
@@ -9261,7 +8210,7 @@
       <c r="T41" s="30"/>
     </row>
     <row r="42" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="17"/>
+      <c r="A42" s="16"/>
       <c r="I42" s="5"/>
       <c r="J42" s="5"/>
       <c r="K42" s="6"/>
@@ -9269,23 +8218,23 @@
       <c r="M42" s="6"/>
       <c r="N42" s="27"/>
       <c r="O42" s="28"/>
-      <c r="P42" s="21"/>
-      <c r="Q42" s="21"/>
-      <c r="R42" s="22"/>
+      <c r="P42" s="20"/>
+      <c r="Q42" s="20"/>
+      <c r="R42" s="21"/>
       <c r="S42" s="22"/>
       <c r="T42" s="22"/>
     </row>
     <row r="43" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="17"/>
+      <c r="A43" s="16"/>
       <c r="N43" s="27"/>
       <c r="P43" s="24"/>
       <c r="Q43" s="24"/>
       <c r="R43" s="25"/>
-      <c r="S43" s="25"/>
-      <c r="T43" s="25"/>
+      <c r="S43" s="22"/>
+      <c r="T43" s="22"/>
     </row>
     <row r="44" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="17"/>
+      <c r="A44" s="16"/>
       <c r="N44" s="27"/>
       <c r="P44" s="5"/>
       <c r="Q44" s="5"/>
@@ -9294,7 +8243,7 @@
       <c r="T44" s="30"/>
     </row>
     <row r="45" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="17"/>
+      <c r="A45" s="16"/>
       <c r="I45" s="5"/>
       <c r="J45" s="5"/>
       <c r="K45" s="6"/>
@@ -9302,14 +8251,14 @@
       <c r="M45" s="6"/>
       <c r="N45" s="27"/>
       <c r="O45" s="28"/>
-      <c r="P45" s="21"/>
-      <c r="Q45" s="21"/>
-      <c r="R45" s="22"/>
+      <c r="P45" s="20"/>
+      <c r="Q45" s="20"/>
+      <c r="R45" s="21"/>
       <c r="S45" s="22"/>
       <c r="T45" s="22"/>
     </row>
     <row r="46" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="17"/>
+      <c r="A46" s="16"/>
       <c r="I46" s="5"/>
       <c r="J46" s="5"/>
       <c r="K46" s="6"/>
@@ -9319,20 +8268,20 @@
       <c r="P46" s="24"/>
       <c r="Q46" s="24"/>
       <c r="R46" s="25"/>
-      <c r="S46" s="25"/>
-      <c r="T46" s="25"/>
+      <c r="S46" s="22"/>
+      <c r="T46" s="22"/>
     </row>
     <row r="47" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="17"/>
-      <c r="I47" s="21" t="n">
+      <c r="A47" s="16"/>
+      <c r="I47" s="20" t="n">
         <f aca="false">VLOOKUP("b5", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="J47" s="21" t="n">
+      <c r="J47" s="20" t="n">
         <f aca="false">VLOOKUP("b5", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="K47" s="22"/>
+      <c r="K47" s="21"/>
       <c r="L47" s="22"/>
       <c r="M47" s="22"/>
       <c r="N47" s="29"/>
@@ -9343,7 +8292,7 @@
       <c r="T47" s="30"/>
     </row>
     <row r="48" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="17"/>
+      <c r="A48" s="16"/>
       <c r="I48" s="24" t="n">
         <f aca="false">VLOOKUP("d5", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
@@ -9353,12 +8302,12 @@
         <v>0</v>
       </c>
       <c r="K48" s="25"/>
-      <c r="L48" s="25"/>
-      <c r="M48" s="25"/>
+      <c r="L48" s="22"/>
+      <c r="M48" s="22"/>
       <c r="T48" s="23"/>
     </row>
     <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="17"/>
+      <c r="A49" s="16"/>
       <c r="I49" s="5"/>
       <c r="J49" s="5"/>
       <c r="K49" s="6"/>
@@ -9367,7 +8316,7 @@
       <c r="T49" s="23"/>
     </row>
     <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="17"/>
+      <c r="A50" s="16"/>
       <c r="I50" s="5"/>
       <c r="J50" s="5"/>
       <c r="K50" s="6"/>
@@ -9376,11 +8325,11 @@
       <c r="T50" s="23"/>
     </row>
     <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="17"/>
+      <c r="A51" s="16"/>
       <c r="T51" s="23"/>
     </row>
     <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="17"/>
+      <c r="A52" s="16"/>
       <c r="B52" s="31"/>
       <c r="C52" s="31"/>
       <c r="D52" s="32"/>
@@ -9405,18 +8354,18 @@
       <c r="A53" s="34" t="s">
         <v>97</v>
       </c>
-      <c r="I53" s="18"/>
-      <c r="J53" s="18"/>
-      <c r="K53" s="19"/>
-      <c r="L53" s="19"/>
-      <c r="M53" s="19"/>
-      <c r="N53" s="18"/>
-      <c r="O53" s="18"/>
-      <c r="P53" s="18"/>
-      <c r="Q53" s="18"/>
-      <c r="R53" s="19"/>
-      <c r="S53" s="19"/>
-      <c r="T53" s="20"/>
+      <c r="I53" s="17"/>
+      <c r="J53" s="17"/>
+      <c r="K53" s="18"/>
+      <c r="L53" s="18"/>
+      <c r="M53" s="18"/>
+      <c r="N53" s="17"/>
+      <c r="O53" s="17"/>
+      <c r="P53" s="17"/>
+      <c r="Q53" s="17"/>
+      <c r="R53" s="18"/>
+      <c r="S53" s="18"/>
+      <c r="T53" s="19"/>
     </row>
     <row r="54" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="34"/>
@@ -9449,15 +8398,15 @@
     </row>
     <row r="59" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="34"/>
-      <c r="P59" s="21" t="n">
+      <c r="P59" s="20" t="n">
         <f aca="false">VLOOKUP("w1", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="Q59" s="21" t="n">
+      <c r="Q59" s="20" t="n">
         <f aca="false">VLOOKUP("w1", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="R59" s="22"/>
+      <c r="R59" s="21"/>
       <c r="S59" s="22"/>
       <c r="T59" s="22"/>
     </row>
@@ -9472,8 +8421,8 @@
         <v>0</v>
       </c>
       <c r="R60" s="25"/>
-      <c r="S60" s="25"/>
-      <c r="T60" s="25"/>
+      <c r="S60" s="22"/>
+      <c r="T60" s="22"/>
     </row>
     <row r="61" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="34"/>
@@ -9481,19 +8430,19 @@
       <c r="Q61" s="5"/>
       <c r="R61" s="6"/>
       <c r="S61" s="6"/>
-      <c r="T61" s="22"/>
+      <c r="T61" s="21"/>
     </row>
     <row r="62" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="34"/>
-      <c r="P62" s="21" t="n">
+      <c r="P62" s="20" t="n">
         <f aca="false">VLOOKUP("w3", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="Q62" s="21" t="n">
+      <c r="Q62" s="20" t="n">
         <f aca="false">VLOOKUP("w3", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="R62" s="22"/>
+      <c r="R62" s="21"/>
       <c r="S62" s="22"/>
       <c r="T62" s="22"/>
     </row>
@@ -9508,8 +8457,8 @@
         <v>0</v>
       </c>
       <c r="R63" s="25"/>
-      <c r="S63" s="25"/>
-      <c r="T63" s="25"/>
+      <c r="S63" s="22"/>
+      <c r="T63" s="22"/>
     </row>
     <row r="64" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="34"/>
@@ -9563,17 +8512,17 @@
       <c r="T69" s="33"/>
     </row>
     <row r="70" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="17" t="s">
+      <c r="A70" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="P70" s="18"/>
-      <c r="Q70" s="18"/>
-      <c r="R70" s="19"/>
-      <c r="S70" s="19"/>
-      <c r="T70" s="20"/>
+      <c r="P70" s="17"/>
+      <c r="Q70" s="17"/>
+      <c r="R70" s="18"/>
+      <c r="S70" s="18"/>
+      <c r="T70" s="19"/>
     </row>
     <row r="71" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="17"/>
+      <c r="A71" s="16"/>
       <c r="I71" s="5"/>
       <c r="J71" s="5"/>
       <c r="K71" s="6"/>
@@ -9582,19 +8531,19 @@
       <c r="T71" s="23"/>
     </row>
     <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="17"/>
+      <c r="A72" s="16"/>
       <c r="T72" s="23"/>
     </row>
     <row r="73" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="17"/>
+      <c r="A73" s="16"/>
       <c r="T73" s="23"/>
     </row>
     <row r="74" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="17"/>
+      <c r="A74" s="16"/>
       <c r="T74" s="23"/>
     </row>
     <row r="75" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="17"/>
+      <c r="A75" s="16"/>
       <c r="P75" s="5"/>
       <c r="Q75" s="5"/>
       <c r="R75" s="6"/>
@@ -9602,21 +8551,21 @@
       <c r="T75" s="30"/>
     </row>
     <row r="76" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="17"/>
-      <c r="P76" s="21" t="n">
+      <c r="A76" s="16"/>
+      <c r="P76" s="20" t="n">
         <f aca="false">VLOOKUP("g1", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="Q76" s="21" t="n">
+      <c r="Q76" s="20" t="n">
         <f aca="false">VLOOKUP("g1", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="R76" s="22"/>
+      <c r="R76" s="21"/>
       <c r="S76" s="22"/>
       <c r="T76" s="22"/>
     </row>
     <row r="77" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="17"/>
+      <c r="A77" s="16"/>
       <c r="P77" s="24" t="n">
         <f aca="false">VLOOKUP("g2", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
@@ -9626,11 +8575,11 @@
         <v>0</v>
       </c>
       <c r="R77" s="25"/>
-      <c r="S77" s="25"/>
-      <c r="T77" s="25"/>
+      <c r="S77" s="22"/>
+      <c r="T77" s="22"/>
     </row>
     <row r="78" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="17"/>
+      <c r="A78" s="16"/>
       <c r="P78" s="5"/>
       <c r="Q78" s="5"/>
       <c r="R78" s="6"/>
@@ -9638,21 +8587,21 @@
       <c r="T78" s="30"/>
     </row>
     <row r="79" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="17"/>
-      <c r="P79" s="21" t="n">
+      <c r="A79" s="16"/>
+      <c r="P79" s="20" t="n">
         <f aca="false">VLOOKUP("g3", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
       </c>
-      <c r="Q79" s="21" t="n">
+      <c r="Q79" s="20" t="n">
         <f aca="false">VLOOKUP("g3", quali_results!$A$1:$C$40,3,0)</f>
         <v>0</v>
       </c>
-      <c r="R79" s="22"/>
+      <c r="R79" s="21"/>
       <c r="S79" s="22"/>
       <c r="T79" s="22"/>
     </row>
     <row r="80" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="17"/>
+      <c r="A80" s="16"/>
       <c r="P80" s="24" t="n">
         <f aca="false">VLOOKUP("g4", quali_results!$A$1:$C$40,2,0)</f>
         <v>0</v>
@@ -9662,11 +8611,11 @@
         <v>0</v>
       </c>
       <c r="R80" s="25"/>
-      <c r="S80" s="25"/>
-      <c r="T80" s="25"/>
+      <c r="S80" s="22"/>
+      <c r="T80" s="22"/>
     </row>
     <row r="81" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="17"/>
+      <c r="A81" s="16"/>
       <c r="P81" s="5"/>
       <c r="Q81" s="5"/>
       <c r="R81" s="6"/>
@@ -9674,15 +8623,15 @@
       <c r="T81" s="30"/>
     </row>
     <row r="82" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="17"/>
+      <c r="A82" s="16"/>
       <c r="T82" s="23"/>
     </row>
     <row r="83" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A83" s="17"/>
+      <c r="A83" s="16"/>
       <c r="T83" s="23"/>
     </row>
     <row r="84" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="17"/>
+      <c r="A84" s="16"/>
       <c r="I84" s="5"/>
       <c r="J84" s="5"/>
       <c r="K84" s="6"/>
@@ -9691,11 +8640,11 @@
       <c r="T84" s="23"/>
     </row>
     <row r="85" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="17"/>
+      <c r="A85" s="16"/>
       <c r="T85" s="23"/>
     </row>
     <row r="86" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="17"/>
+      <c r="A86" s="16"/>
       <c r="B86" s="31"/>
       <c r="C86" s="31"/>
       <c r="D86" s="32"/>
@@ -9734,13 +8683,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D27"/>
-  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.92"/>
@@ -9784,7 +8733,7 @@
       <c r="D9" s="38"/>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="16" t="s">
         <v>104</v>
       </c>
       <c r="B10" s="40"/>
@@ -9794,22 +8743,22 @@
       </c>
     </row>
     <row r="11" s="9" customFormat="true" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="16" t="s">
         <v>106</v>
       </c>
       <c r="B11" s="40"/>
       <c r="C11" s="40"/>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="16" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="12" s="9" customFormat="true" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="B12" s="40"/>
-      <c r="C12" s="40"/>
-      <c r="D12" s="17" t="s">
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="16" t="s">
         <v>107</v>
       </c>
     </row>
@@ -9817,9 +8766,9 @@
       <c r="A13" s="42" t="s">
         <v>108</v>
       </c>
-      <c r="B13" s="43"/>
-      <c r="C13" s="43"/>
-      <c r="D13" s="17" t="s">
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="16" t="s">
         <v>108</v>
       </c>
     </row>
@@ -9864,7 +8813,7 @@
       <c r="D23" s="38"/>
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="16" t="s">
         <v>104</v>
       </c>
       <c r="B24" s="40"/>
@@ -9874,22 +8823,22 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17" t="s">
+      <c r="A25" s="16" t="s">
         <v>106</v>
       </c>
       <c r="B25" s="40"/>
       <c r="C25" s="40"/>
-      <c r="D25" s="17" t="s">
+      <c r="D25" s="16" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17" t="s">
+      <c r="A26" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="B26" s="40"/>
-      <c r="C26" s="40"/>
-      <c r="D26" s="17" t="s">
+      <c r="B26" s="22"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="16" t="s">
         <v>107</v>
       </c>
     </row>
@@ -9899,7 +8848,7 @@
       </c>
       <c r="B27" s="43"/>
       <c r="C27" s="43"/>
-      <c r="D27" s="17" t="s">
+      <c r="D27" s="16" t="s">
         <v>108</v>
       </c>
     </row>

</xml_diff>